<commit_message>
chagemment de la synthese hebdomadaire de fiche de paie
</commit_message>
<xml_diff>
--- a/public/PLAN.xlsx
+++ b/public/PLAN.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\log_project\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{52CE9F4B-C522-47E0-84A7-0F2A6AC84B10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8F2FFDD-A311-4AA0-8260-614EA14C2988}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="19425" windowHeight="10305" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLAN COMPTABLE" sheetId="1" r:id="rId1"/>
@@ -20,23 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="659" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="661" uniqueCount="339">
   <si>
     <t>Comptes</t>
   </si>
@@ -1050,6 +1039,9 @@
   </si>
   <si>
     <t>Transfert de charge</t>
+  </si>
+  <si>
+    <t>Impôt général sur le bénefice</t>
   </si>
 </sst>
 </file>
@@ -1057,9 +1049,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1197,10 +1189,10 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1215,6 +1207,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="20 % - Accent1 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -1524,15 +1517,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C333"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <dimension ref="A1:C334"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.42578125" customWidth="1"/>
-    <col min="2" max="2" width="66.42578125" customWidth="1"/>
-    <col min="3" max="3" width="19.42578125" customWidth="1"/>
+    <col min="1" max="1" width="19.453125" customWidth="1"/>
+    <col min="2" max="2" width="66.453125" customWidth="1"/>
+    <col min="3" max="3" width="19.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18.75">
+    <row r="1" spans="1:3" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -1541,7 +1534,7 @@
       </c>
       <c r="C1" s="6"/>
     </row>
-    <row r="2" spans="1:3" ht="18.75">
+    <row r="2" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A2" s="1">
         <v>1010000000</v>
       </c>
@@ -1552,7 +1545,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="18.75">
+    <row r="3" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A3" s="1">
         <v>1040000001</v>
       </c>
@@ -1563,7 +1556,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="18.75">
+    <row r="4" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A4" s="1">
         <v>1040000002</v>
       </c>
@@ -1574,7 +1567,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="18.75">
+    <row r="5" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A5" s="1">
         <v>1040000003</v>
       </c>
@@ -1585,7 +1578,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="18.75">
+    <row r="6" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A6" s="1">
         <v>1040000004</v>
       </c>
@@ -1596,7 +1589,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="18.75">
+    <row r="7" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A7" s="1">
         <v>1040000005</v>
       </c>
@@ -1607,7 +1600,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="18.75">
+    <row r="8" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A8" s="1">
         <v>1851000000</v>
       </c>
@@ -1616,7 +1609,7 @@
       </c>
       <c r="C8" s="1"/>
     </row>
-    <row r="9" spans="1:3" ht="18.75">
+    <row r="9" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A9" s="1">
         <v>1852000000</v>
       </c>
@@ -1625,7 +1618,7 @@
       </c>
       <c r="C9" s="1"/>
     </row>
-    <row r="10" spans="1:3" ht="18.75">
+    <row r="10" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A10" s="1">
         <v>1861000000</v>
       </c>
@@ -1634,7 +1627,7 @@
       </c>
       <c r="C10" s="1"/>
     </row>
-    <row r="11" spans="1:3" ht="18.75">
+    <row r="11" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A11" s="1">
         <v>1862000000</v>
       </c>
@@ -1643,7 +1636,7 @@
       </c>
       <c r="C11" s="1"/>
     </row>
-    <row r="12" spans="1:3" ht="18.75">
+    <row r="12" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A12" s="1">
         <v>1871000000</v>
       </c>
@@ -1652,7 +1645,7 @@
       </c>
       <c r="C12" s="1"/>
     </row>
-    <row r="13" spans="1:3" ht="18.75">
+    <row r="13" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A13" s="1">
         <v>1872000000</v>
       </c>
@@ -1661,7 +1654,7 @@
       </c>
       <c r="C13" s="1"/>
     </row>
-    <row r="14" spans="1:3" ht="18.75">
+    <row r="14" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A14" s="1">
         <v>2193000001</v>
       </c>
@@ -1672,7 +1665,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="18.75">
+    <row r="15" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A15" s="1">
         <v>2193000002</v>
       </c>
@@ -1683,7 +1676,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="18.75">
+    <row r="16" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A16" s="1">
         <v>2193000003</v>
       </c>
@@ -1694,7 +1687,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="18.75">
+    <row r="17" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A17" s="1">
         <v>2193000004</v>
       </c>
@@ -1705,7 +1698,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="18.75">
+    <row r="18" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A18" s="1">
         <v>2230000000</v>
       </c>
@@ -1716,7 +1709,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="18.75">
+    <row r="19" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A19" s="1">
         <v>2251000000</v>
       </c>
@@ -1727,7 +1720,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="18.75">
+    <row r="20" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A20" s="1">
         <v>2313000000</v>
       </c>
@@ -1738,7 +1731,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="18.75">
+    <row r="21" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A21" s="1">
         <v>2351000000</v>
       </c>
@@ -1749,7 +1742,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="18.75">
+    <row r="22" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A22" s="1">
         <v>2358000000</v>
       </c>
@@ -1760,7 +1753,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="18.75">
+    <row r="23" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A23" s="1">
         <v>2421000001</v>
       </c>
@@ -1771,7 +1764,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="18.75">
+    <row r="24" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A24" s="1">
         <v>2421000021</v>
       </c>
@@ -1782,7 +1775,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="18.75">
+    <row r="25" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A25" s="1">
         <v>2421000022</v>
       </c>
@@ -1793,7 +1786,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="18.75">
+    <row r="26" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A26" s="1">
         <v>2421000003</v>
       </c>
@@ -1804,7 +1797,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="18.75">
+    <row r="27" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A27" s="1">
         <v>2421000004</v>
       </c>
@@ -1815,7 +1808,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="18.75">
+    <row r="28" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A28" s="1">
         <v>2441000001</v>
       </c>
@@ -1826,7 +1819,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="18.75">
+    <row r="29" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A29" s="1">
         <v>2441000002</v>
       </c>
@@ -1837,7 +1830,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="18.75">
+    <row r="30" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A30" s="1">
         <v>2442000001</v>
       </c>
@@ -1848,7 +1841,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="18.75">
+    <row r="31" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A31" s="1">
         <v>2442000002</v>
       </c>
@@ -1859,7 +1852,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="18.75">
+    <row r="32" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A32" s="1">
         <v>2442000003</v>
       </c>
@@ -1870,7 +1863,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="18.75">
+    <row r="33" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A33" s="1">
         <v>2444000001</v>
       </c>
@@ -1881,7 +1874,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="18.75">
+    <row r="34" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A34" s="1">
         <v>2444000002</v>
       </c>
@@ -1892,7 +1885,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="18.75">
+    <row r="35" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A35" s="1">
         <v>2444000003</v>
       </c>
@@ -1903,7 +1896,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="18.75">
+    <row r="36" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A36" s="1">
         <v>2444000004</v>
       </c>
@@ -1914,7 +1907,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="18.75">
+    <row r="37" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A37" s="1">
         <v>2444000005</v>
       </c>
@@ -1925,7 +1918,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="18.75">
+    <row r="38" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A38" s="1">
         <v>2444000006</v>
       </c>
@@ -1936,7 +1929,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="18.75">
+    <row r="39" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A39" s="1">
         <v>2444000007</v>
       </c>
@@ -1947,7 +1940,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="18.75">
+    <row r="40" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A40" s="1">
         <v>2444000008</v>
       </c>
@@ -1958,7 +1951,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="18.75">
+    <row r="41" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A41" s="1">
         <v>2450000001</v>
       </c>
@@ -1969,7 +1962,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="18.75">
+    <row r="42" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A42" s="1">
         <v>2450000002</v>
       </c>
@@ -1980,7 +1973,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="18.75">
+    <row r="43" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A43" s="1">
         <v>2450000003</v>
       </c>
@@ -1991,7 +1984,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="18.75">
+    <row r="44" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A44" s="1">
         <v>2451000001</v>
       </c>
@@ -2002,7 +1995,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="45" spans="1:3" ht="18.75">
+    <row r="45" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A45" s="1">
         <v>2451000002</v>
       </c>
@@ -2013,7 +2006,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="18.75">
+    <row r="46" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A46" s="1">
         <v>2451000003</v>
       </c>
@@ -2024,7 +2017,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="47" spans="1:3" ht="18.75">
+    <row r="47" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A47" s="1">
         <v>2451000004</v>
       </c>
@@ -2035,7 +2028,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="48" spans="1:3" ht="18.75">
+    <row r="48" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A48" s="1">
         <v>2810000001</v>
       </c>
@@ -2046,7 +2039,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="18.75">
+    <row r="49" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A49" s="1">
         <v>2810000002</v>
       </c>
@@ -2057,7 +2050,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="50" spans="1:3" ht="18.75">
+    <row r="50" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A50" s="1">
         <v>2810000003</v>
       </c>
@@ -2068,7 +2061,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="51" spans="1:3" ht="18.75">
+    <row r="51" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A51" s="1">
         <v>2810000004</v>
       </c>
@@ -2079,7 +2072,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="52" spans="1:3" ht="18.75">
+    <row r="52" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A52" s="1">
         <v>2840000001</v>
       </c>
@@ -2090,7 +2083,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="53" spans="1:3" ht="18.75">
+    <row r="53" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A53" s="1">
         <v>2840000002</v>
       </c>
@@ -2101,7 +2094,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="54" spans="1:3" ht="18.75">
+    <row r="54" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A54" s="1">
         <v>2840000003</v>
       </c>
@@ -2112,7 +2105,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="55" spans="1:3" ht="18.75">
+    <row r="55" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A55" s="1">
         <v>2840000004</v>
       </c>
@@ -2123,7 +2116,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="56" spans="1:3" ht="18.75">
+    <row r="56" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A56" s="1">
         <v>2840000005</v>
       </c>
@@ -2134,7 +2127,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="57" spans="1:3" ht="18.75">
+    <row r="57" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A57" s="1">
         <v>2840000006</v>
       </c>
@@ -2145,7 +2138,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="58" spans="1:3" ht="18.75">
+    <row r="58" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A58" s="1">
         <v>2840000007</v>
       </c>
@@ -2156,7 +2149,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="59" spans="1:3" ht="18.75">
+    <row r="59" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A59" s="1">
         <v>2840000008</v>
       </c>
@@ -2167,7 +2160,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="60" spans="1:3" ht="18.75">
+    <row r="60" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A60" s="1">
         <v>2840000009</v>
       </c>
@@ -2178,7 +2171,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="61" spans="1:3" ht="18.75">
+    <row r="61" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A61" s="1">
         <v>2840000010</v>
       </c>
@@ -2189,7 +2182,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="62" spans="1:3" ht="18.75">
+    <row r="62" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A62" s="1">
         <v>2840000011</v>
       </c>
@@ -2200,7 +2193,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="63" spans="1:3" ht="18.75">
+    <row r="63" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A63" s="1">
         <v>2840000012</v>
       </c>
@@ -2211,7 +2204,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="64" spans="1:3" ht="18.75">
+    <row r="64" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A64" s="1">
         <v>2840000013</v>
       </c>
@@ -2222,7 +2215,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="65" spans="1:3" ht="18.75">
+    <row r="65" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A65" s="1">
         <v>2840000014</v>
       </c>
@@ -2233,7 +2226,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="66" spans="1:3" ht="18.75">
+    <row r="66" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A66" s="1">
         <v>2840000015</v>
       </c>
@@ -2244,7 +2237,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="67" spans="1:3" ht="18.75">
+    <row r="67" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A67" s="1">
         <v>2840000016</v>
       </c>
@@ -2255,7 +2248,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="68" spans="1:3" ht="18.75">
+    <row r="68" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A68" s="1">
         <v>2840000017</v>
       </c>
@@ -2266,7 +2259,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="69" spans="1:3" ht="18.75">
+    <row r="69" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A69" s="1">
         <v>2840000018</v>
       </c>
@@ -2277,7 +2270,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="70" spans="1:3" ht="18.75">
+    <row r="70" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A70" s="1">
         <v>2840000019</v>
       </c>
@@ -2288,7 +2281,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="71" spans="1:3" ht="18.75">
+    <row r="71" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A71" s="1">
         <v>2840000020</v>
       </c>
@@ -2299,7 +2292,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="72" spans="1:3" ht="18.75">
+    <row r="72" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A72" s="1">
         <v>2840000021</v>
       </c>
@@ -2310,7 +2303,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="73" spans="1:3" ht="18.75">
+    <row r="73" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A73" s="1">
         <v>2840000022</v>
       </c>
@@ -2321,7 +2314,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="74" spans="1:3" ht="18.75">
+    <row r="74" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A74" s="1">
         <v>2840000023</v>
       </c>
@@ -2332,7 +2325,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="75" spans="1:3" ht="18.75">
+    <row r="75" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A75" s="1">
         <v>2840000024</v>
       </c>
@@ -2343,7 +2336,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="76" spans="1:3" ht="18.75">
+    <row r="76" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A76" s="1">
         <v>2840000025</v>
       </c>
@@ -2354,7 +2347,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="77" spans="1:3" ht="18.75">
+    <row r="77" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A77" s="1">
         <v>2840000026</v>
       </c>
@@ -2365,7 +2358,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="78" spans="1:3" ht="18.75">
+    <row r="78" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A78" s="1">
         <v>2840000027</v>
       </c>
@@ -2376,7 +2369,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="79" spans="1:3" ht="18.75">
+    <row r="79" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A79" s="1">
         <v>2840000028</v>
       </c>
@@ -2387,7 +2380,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="80" spans="1:3" ht="18.75">
+    <row r="80" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A80" s="1">
         <v>3340000001</v>
       </c>
@@ -2398,7 +2391,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="81" spans="1:3" ht="18.75">
+    <row r="81" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A81" s="1">
         <v>3340000002</v>
       </c>
@@ -2409,7 +2402,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="82" spans="1:3" ht="18.75">
+    <row r="82" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A82" s="1">
         <v>3340000003</v>
       </c>
@@ -2420,7 +2413,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="83" spans="1:3" ht="18.75">
+    <row r="83" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A83" s="1">
         <v>3340000004</v>
       </c>
@@ -2431,7 +2424,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="84" spans="1:3" ht="18.75">
+    <row r="84" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A84" s="1">
         <v>3340000005</v>
       </c>
@@ -2442,7 +2435,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="85" spans="1:3" ht="18.75">
+    <row r="85" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A85" s="1">
         <v>3340000006</v>
       </c>
@@ -2453,7 +2446,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="86" spans="1:3" ht="18.75">
+    <row r="86" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A86" s="1">
         <v>3340000007</v>
       </c>
@@ -2464,7 +2457,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="87" spans="1:3" ht="18.75">
+    <row r="87" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A87" s="1">
         <v>3340000008</v>
       </c>
@@ -2475,7 +2468,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="88" spans="1:3" ht="18.75">
+    <row r="88" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A88" s="1">
         <v>3340000009</v>
       </c>
@@ -2486,7 +2479,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="89" spans="1:3" ht="18.75">
+    <row r="89" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A89" s="1">
         <v>3340000010</v>
       </c>
@@ -2497,7 +2490,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="90" spans="1:3" ht="18.75">
+    <row r="90" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A90" s="1">
         <v>3340000011</v>
       </c>
@@ -2508,7 +2501,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="91" spans="1:3" ht="18.75">
+    <row r="91" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A91" s="1">
         <v>3340000012</v>
       </c>
@@ -2519,7 +2512,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="92" spans="1:3" ht="18.75">
+    <row r="92" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A92" s="1">
         <v>3340000013</v>
       </c>
@@ -2530,7 +2523,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="93" spans="1:3" ht="18.75">
+    <row r="93" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A93" s="1">
         <v>3340000014</v>
       </c>
@@ -2541,7 +2534,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="94" spans="1:3" ht="18.75">
+    <row r="94" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A94" s="1">
         <v>3340000015</v>
       </c>
@@ -2552,7 +2545,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="95" spans="1:3" ht="18.75">
+    <row r="95" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A95" s="1">
         <v>3340000016</v>
       </c>
@@ -2563,7 +2556,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="96" spans="1:3" ht="18.75">
+    <row r="96" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A96" s="1">
         <v>3340000017</v>
       </c>
@@ -2574,7 +2567,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="97" spans="1:3" ht="18.75">
+    <row r="97" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A97" s="1">
         <v>3340000018</v>
       </c>
@@ -2585,7 +2578,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="98" spans="1:3" ht="18.75">
+    <row r="98" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A98" s="1">
         <v>3340000019</v>
       </c>
@@ -2596,7 +2589,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="99" spans="1:3" ht="18.75">
+    <row r="99" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A99" s="1">
         <v>3340000020</v>
       </c>
@@ -2607,7 +2600,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="100" spans="1:3" ht="18.75">
+    <row r="100" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A100" s="1">
         <v>3340000021</v>
       </c>
@@ -2618,7 +2611,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="101" spans="1:3" ht="18.75">
+    <row r="101" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A101" s="1">
         <v>3340000022</v>
       </c>
@@ -2629,7 +2622,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="102" spans="1:3" ht="18.75">
+    <row r="102" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A102" s="1">
         <v>3340000023</v>
       </c>
@@ -2640,7 +2633,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="103" spans="1:3" ht="18.75">
+    <row r="103" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A103" s="1">
         <v>3340000024</v>
       </c>
@@ -2651,7 +2644,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="104" spans="1:3" ht="18.75">
+    <row r="104" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A104" s="1">
         <v>3340000025</v>
       </c>
@@ -2662,7 +2655,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="105" spans="1:3" ht="18.75">
+    <row r="105" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A105" s="1">
         <v>3340000026</v>
       </c>
@@ -2673,7 +2666,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="106" spans="1:3" ht="18.75">
+    <row r="106" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A106" s="1">
         <v>3340000027</v>
       </c>
@@ -2684,7 +2677,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="107" spans="1:3" ht="18.75">
+    <row r="107" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A107" s="1">
         <v>3340000028</v>
       </c>
@@ -2695,7 +2688,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="108" spans="1:3" ht="18.75">
+    <row r="108" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A108" s="1">
         <v>3340000029</v>
       </c>
@@ -2706,7 +2699,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="109" spans="1:3" ht="18.75">
+    <row r="109" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A109" s="1">
         <v>3340000030</v>
       </c>
@@ -2717,7 +2710,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="110" spans="1:3" ht="18.75">
+    <row r="110" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A110" s="1">
         <v>3340000031</v>
       </c>
@@ -2728,7 +2721,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="111" spans="1:3" ht="18.75">
+    <row r="111" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A111" s="1">
         <v>3340000032</v>
       </c>
@@ -2739,7 +2732,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="112" spans="1:3" ht="18.75">
+    <row r="112" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A112" s="1">
         <v>3340000033</v>
       </c>
@@ -2750,7 +2743,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="113" spans="1:3" ht="18.75">
+    <row r="113" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A113" s="1">
         <v>3340000034</v>
       </c>
@@ -2761,7 +2754,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="114" spans="1:3" ht="18.75">
+    <row r="114" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A114" s="1">
         <v>3340000035</v>
       </c>
@@ -2772,7 +2765,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="115" spans="1:3" ht="18.75">
+    <row r="115" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A115" s="1">
         <v>3340000036</v>
       </c>
@@ -2783,7 +2776,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="116" spans="1:3" ht="18.75">
+    <row r="116" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A116" s="1">
         <v>3340000037</v>
       </c>
@@ -2794,7 +2787,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="117" spans="1:3" ht="18.75">
+    <row r="117" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A117" s="1">
         <v>3340000038</v>
       </c>
@@ -2805,7 +2798,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="118" spans="1:3" ht="18.75">
+    <row r="118" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A118" s="1">
         <v>3340000039</v>
       </c>
@@ -2816,7 +2809,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="119" spans="1:3" ht="18.75">
+    <row r="119" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A119" s="3">
         <v>3340000040</v>
       </c>
@@ -2827,7 +2820,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="120" spans="1:3" ht="18.75">
+    <row r="120" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A120" s="1">
         <v>3340000041</v>
       </c>
@@ -2838,7 +2831,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="121" spans="1:3" ht="18.75">
+    <row r="121" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A121" s="3">
         <v>3340000042</v>
       </c>
@@ -2849,7 +2842,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="122" spans="1:3" ht="18.75">
+    <row r="122" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A122" s="1">
         <v>4010000001</v>
       </c>
@@ -2860,7 +2853,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="123" spans="1:3" ht="18.75">
+    <row r="123" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A123" s="1">
         <v>4010000021</v>
       </c>
@@ -2871,7 +2864,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="124" spans="1:3" ht="18.75">
+    <row r="124" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A124" s="1">
         <v>4010000022</v>
       </c>
@@ -2882,7 +2875,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="125" spans="1:3" ht="18.75">
+    <row r="125" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A125" s="1">
         <v>4010000003</v>
       </c>
@@ -2893,7 +2886,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="126" spans="1:3" ht="18.75">
+    <row r="126" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A126" s="1">
         <v>4010000004</v>
       </c>
@@ -2904,7 +2897,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="127" spans="1:3" ht="18.75">
+    <row r="127" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A127" s="1">
         <v>4010000005</v>
       </c>
@@ -2915,7 +2908,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="128" spans="1:3" ht="18.75">
+    <row r="128" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A128" s="1">
         <v>4010000006</v>
       </c>
@@ -2926,7 +2919,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="129" spans="1:3" ht="18.75">
+    <row r="129" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A129" s="1">
         <v>4010000007</v>
       </c>
@@ -2937,7 +2930,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="130" spans="1:3" ht="18.75">
+    <row r="130" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A130" s="1">
         <v>4010000008</v>
       </c>
@@ -2948,7 +2941,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="131" spans="1:3" ht="18.75">
+    <row r="131" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A131" s="1">
         <v>4010000009</v>
       </c>
@@ -2959,7 +2952,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="132" spans="1:3" ht="18.75">
+    <row r="132" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A132" s="1">
         <v>4010000010</v>
       </c>
@@ -2970,7 +2963,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="133" spans="1:3" ht="18.75">
+    <row r="133" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A133" s="1">
         <v>4040000000</v>
       </c>
@@ -2981,7 +2974,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="134" spans="1:3" ht="18.75">
+    <row r="134" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A134" s="1">
         <v>4090000000</v>
       </c>
@@ -2992,7 +2985,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="135" spans="1:3" ht="18.75">
+    <row r="135" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A135" s="1">
         <v>4110000000</v>
       </c>
@@ -3003,7 +2996,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="136" spans="1:3" ht="18.75">
+    <row r="136" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A136" s="1">
         <v>4210000000</v>
       </c>
@@ -3014,7 +3007,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="137" spans="1:3" ht="18.75">
+    <row r="137" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A137" s="1">
         <v>4211000000</v>
       </c>
@@ -3025,7 +3018,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="138" spans="1:3" ht="18.75">
+    <row r="138" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A138" s="1">
         <v>4220000000</v>
       </c>
@@ -3036,7 +3029,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="139" spans="1:3" ht="18.75">
+    <row r="139" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A139" s="1">
         <v>4474000000</v>
       </c>
@@ -3047,7 +3040,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="140" spans="1:3" ht="18.75">
+    <row r="140" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A140" s="1">
         <v>4475000000</v>
       </c>
@@ -3058,7 +3051,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="141" spans="1:3" ht="18.75">
+    <row r="141" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A141" s="1">
         <v>4471000000</v>
       </c>
@@ -3069,7 +3062,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="142" spans="1:3" ht="18.75">
+    <row r="142" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A142" s="1">
         <v>4472000000</v>
       </c>
@@ -3080,7 +3073,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="143" spans="1:3" ht="18.75">
+    <row r="143" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A143" s="4">
         <v>4620000001</v>
       </c>
@@ -3091,7 +3084,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="144" spans="1:3" ht="18.75">
+    <row r="144" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A144" s="4">
         <v>4620000002</v>
       </c>
@@ -3102,7 +3095,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="145" spans="1:3" ht="18.75">
+    <row r="145" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A145" s="4">
         <v>4620000003</v>
       </c>
@@ -3113,7 +3106,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="146" spans="1:3" ht="18.75">
+    <row r="146" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A146" s="4">
         <v>4620000004</v>
       </c>
@@ -3124,7 +3117,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="147" spans="1:3" ht="18.75">
+    <row r="147" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A147" s="4">
         <v>4620000005</v>
       </c>
@@ -3135,7 +3128,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="148" spans="1:3" ht="18.75">
+    <row r="148" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A148" s="4">
         <v>4712000000</v>
       </c>
@@ -3146,7 +3139,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="149" spans="1:3" ht="18.75">
+    <row r="149" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A149" s="4">
         <v>4722000000</v>
       </c>
@@ -3157,7 +3150,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="150" spans="1:3" ht="18.75">
+    <row r="150" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A150" s="1">
         <v>5200000000</v>
       </c>
@@ -3168,7 +3161,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="151" spans="1:3" ht="18.75">
+    <row r="151" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A151" s="1">
         <v>5700000000</v>
       </c>
@@ -3179,7 +3172,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="152" spans="1:3" ht="18.75">
+    <row r="152" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A152" s="1">
         <v>5810000000</v>
       </c>
@@ -3188,7 +3181,7 @@
       </c>
       <c r="C152" s="1"/>
     </row>
-    <row r="153" spans="1:3" ht="18.75">
+    <row r="153" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A153" s="1">
         <v>6033000001</v>
       </c>
@@ -3199,7 +3192,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="154" spans="1:3" ht="18.75">
+    <row r="154" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A154" s="1">
         <v>6033000002</v>
       </c>
@@ -3210,7 +3203,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="155" spans="1:3" ht="18.75">
+    <row r="155" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A155" s="1">
         <v>6033000003</v>
       </c>
@@ -3221,7 +3214,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="156" spans="1:3" ht="18.75">
+    <row r="156" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A156" s="1">
         <v>6033000004</v>
       </c>
@@ -3232,7 +3225,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="157" spans="1:3" ht="18.75">
+    <row r="157" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A157" s="1">
         <v>6033000005</v>
       </c>
@@ -3243,7 +3236,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="158" spans="1:3" ht="18.75">
+    <row r="158" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A158" s="1">
         <v>6033000006</v>
       </c>
@@ -3254,7 +3247,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="159" spans="1:3" ht="18.75">
+    <row r="159" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A159" s="1">
         <v>6033000007</v>
       </c>
@@ -3265,7 +3258,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="160" spans="1:3" ht="18.75">
+    <row r="160" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A160" s="1">
         <v>6033000008</v>
       </c>
@@ -3276,7 +3269,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="161" spans="1:3" ht="18.75">
+    <row r="161" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A161" s="1">
         <v>6033000009</v>
       </c>
@@ -3287,7 +3280,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="162" spans="1:3" ht="18.75">
+    <row r="162" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A162" s="1">
         <v>6033000010</v>
       </c>
@@ -3298,7 +3291,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="163" spans="1:3" ht="18.75">
+    <row r="163" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A163" s="1">
         <v>6033000011</v>
       </c>
@@ -3309,7 +3302,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="164" spans="1:3" ht="18.75">
+    <row r="164" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A164" s="1">
         <v>6033000012</v>
       </c>
@@ -3320,7 +3313,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="165" spans="1:3" ht="18.75">
+    <row r="165" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A165" s="1">
         <v>6033000013</v>
       </c>
@@ -3331,7 +3324,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="166" spans="1:3" ht="18.75">
+    <row r="166" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A166" s="1">
         <v>6033000014</v>
       </c>
@@ -3342,7 +3335,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="167" spans="1:3" ht="18.75">
+    <row r="167" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A167" s="1">
         <v>6033000015</v>
       </c>
@@ -3353,7 +3346,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="168" spans="1:3" ht="18.75">
+    <row r="168" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A168" s="1">
         <v>6033000016</v>
       </c>
@@ -3364,7 +3357,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="169" spans="1:3" ht="18.75">
+    <row r="169" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A169" s="1">
         <v>6033000017</v>
       </c>
@@ -3375,7 +3368,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="170" spans="1:3" ht="18.75">
+    <row r="170" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A170" s="1">
         <v>6033000018</v>
       </c>
@@ -3386,7 +3379,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="171" spans="1:3" ht="18.75">
+    <row r="171" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A171" s="1">
         <v>6033000019</v>
       </c>
@@ -3397,7 +3390,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="172" spans="1:3" ht="18.75">
+    <row r="172" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A172" s="1">
         <v>6033000020</v>
       </c>
@@ -3408,7 +3401,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="173" spans="1:3" ht="18.75">
+    <row r="173" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A173" s="1">
         <v>6033000021</v>
       </c>
@@ -3419,7 +3412,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="174" spans="1:3" ht="18.75">
+    <row r="174" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A174" s="1">
         <v>6033000022</v>
       </c>
@@ -3430,7 +3423,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="175" spans="1:3" ht="18.75">
+    <row r="175" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A175" s="1">
         <v>6033000023</v>
       </c>
@@ -3441,7 +3434,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="176" spans="1:3" ht="18.75">
+    <row r="176" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A176" s="1">
         <v>6033000024</v>
       </c>
@@ -3452,7 +3445,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="177" spans="1:3" ht="18.75">
+    <row r="177" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A177" s="1">
         <v>6033000025</v>
       </c>
@@ -3463,7 +3456,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="178" spans="1:3" ht="18.75">
+    <row r="178" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A178" s="1">
         <v>6033000026</v>
       </c>
@@ -3474,7 +3467,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="179" spans="1:3" ht="18.75">
+    <row r="179" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A179" s="1">
         <v>6033000027</v>
       </c>
@@ -3485,7 +3478,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="180" spans="1:3" ht="18.75">
+    <row r="180" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A180" s="1">
         <v>6033000028</v>
       </c>
@@ -3496,7 +3489,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="181" spans="1:3" ht="18.75">
+    <row r="181" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A181" s="1">
         <v>6033000029</v>
       </c>
@@ -3507,7 +3500,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="182" spans="1:3" ht="18.75">
+    <row r="182" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A182" s="1">
         <v>6033000030</v>
       </c>
@@ -3518,7 +3511,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="183" spans="1:3" ht="18.75">
+    <row r="183" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A183" s="1">
         <v>6033000031</v>
       </c>
@@ -3529,7 +3522,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="184" spans="1:3" ht="18.75">
+    <row r="184" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A184" s="1">
         <v>6033000032</v>
       </c>
@@ -3540,7 +3533,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="185" spans="1:3" ht="18.75">
+    <row r="185" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A185" s="1">
         <v>6033000033</v>
       </c>
@@ -3551,7 +3544,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="186" spans="1:3" ht="18.75">
+    <row r="186" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A186" s="1">
         <v>6033000034</v>
       </c>
@@ -3562,7 +3555,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="187" spans="1:3" ht="18.75">
+    <row r="187" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A187" s="1">
         <v>6033000035</v>
       </c>
@@ -3573,7 +3566,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="188" spans="1:3" ht="18.75">
+    <row r="188" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A188" s="1">
         <v>6033000036</v>
       </c>
@@ -3584,7 +3577,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="189" spans="1:3" ht="18.75">
+    <row r="189" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A189" s="1">
         <v>6033000037</v>
       </c>
@@ -3595,7 +3588,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="190" spans="1:3" ht="18.75">
+    <row r="190" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A190" s="1">
         <v>6033000038</v>
       </c>
@@ -3606,7 +3599,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="191" spans="1:3" ht="18.75">
+    <row r="191" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A191" s="3">
         <v>6033000039</v>
       </c>
@@ -3617,7 +3610,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="192" spans="1:3" ht="18.75">
+    <row r="192" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A192" s="1">
         <v>6033000040</v>
       </c>
@@ -3628,7 +3621,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="193" spans="1:3" ht="18.75">
+    <row r="193" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A193" s="3">
         <v>6033000041</v>
       </c>
@@ -3639,7 +3632,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="194" spans="1:3" ht="18.75">
+    <row r="194" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A194" s="1">
         <v>6047000001</v>
       </c>
@@ -3650,7 +3643,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="195" spans="1:3" ht="18.75">
+    <row r="195" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A195" s="1">
         <v>6047000002</v>
       </c>
@@ -3661,7 +3654,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="196" spans="1:3" ht="18.75">
+    <row r="196" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A196" s="1">
         <v>6047000003</v>
       </c>
@@ -3672,7 +3665,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="197" spans="1:3" ht="18.75">
+    <row r="197" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A197" s="1">
         <v>6047000004</v>
       </c>
@@ -3683,7 +3676,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="198" spans="1:3" ht="18.75">
+    <row r="198" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A198" s="1">
         <v>6047000005</v>
       </c>
@@ -3694,7 +3687,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="199" spans="1:3" ht="18.75">
+    <row r="199" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A199" s="1">
         <v>6047000006</v>
       </c>
@@ -3705,7 +3698,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="200" spans="1:3" ht="18.75">
+    <row r="200" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A200" s="1">
         <v>6047000007</v>
       </c>
@@ -3716,7 +3709,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="201" spans="1:3" ht="18.75">
+    <row r="201" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A201" s="1">
         <v>6047000008</v>
       </c>
@@ -3727,7 +3720,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="202" spans="1:3" ht="18.75">
+    <row r="202" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A202" s="1">
         <v>6047000009</v>
       </c>
@@ -3738,7 +3731,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="203" spans="1:3" ht="18.75">
+    <row r="203" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A203" s="1">
         <v>6047000010</v>
       </c>
@@ -3749,7 +3742,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="204" spans="1:3" ht="18.75">
+    <row r="204" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A204" s="1">
         <v>6047000011</v>
       </c>
@@ -3760,7 +3753,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="205" spans="1:3" ht="18.75">
+    <row r="205" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A205" s="1">
         <v>6047000012</v>
       </c>
@@ -3771,7 +3764,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="206" spans="1:3" ht="18.75">
+    <row r="206" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A206" s="1">
         <v>6055000001</v>
       </c>
@@ -3782,7 +3775,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="207" spans="1:3" ht="18.75">
+    <row r="207" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A207" s="1">
         <v>6055000002</v>
       </c>
@@ -3793,7 +3786,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="208" spans="1:3" ht="18.75">
+    <row r="208" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A208" s="1">
         <v>6055000003</v>
       </c>
@@ -3804,7 +3797,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="209" spans="1:3" ht="18.75">
+    <row r="209" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A209" s="1">
         <v>6055000004</v>
       </c>
@@ -3815,7 +3808,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="210" spans="1:3" ht="18.75">
+    <row r="210" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A210" s="1">
         <v>6055000005</v>
       </c>
@@ -3826,7 +3819,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="211" spans="1:3" ht="18.75">
+    <row r="211" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A211" s="1">
         <v>6055000006</v>
       </c>
@@ -3837,7 +3830,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="212" spans="1:3" ht="18.75">
+    <row r="212" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A212" s="1">
         <v>6055000007</v>
       </c>
@@ -3848,7 +3841,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="213" spans="1:3" ht="18.75">
+    <row r="213" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A213" s="1">
         <v>6055000008</v>
       </c>
@@ -3859,7 +3852,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="214" spans="1:3" ht="18.75">
+    <row r="214" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A214" s="1">
         <v>6055000009</v>
       </c>
@@ -3870,7 +3863,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="215" spans="1:3" ht="18.75">
+    <row r="215" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A215" s="1">
         <v>6055000010</v>
       </c>
@@ -3881,7 +3874,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="216" spans="1:3" ht="18.75">
+    <row r="216" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A216" s="1">
         <v>6055000011</v>
       </c>
@@ -3892,7 +3885,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="217" spans="1:3" ht="18.75">
+    <row r="217" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A217" s="1">
         <v>6055000012</v>
       </c>
@@ -3903,7 +3896,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="218" spans="1:3" ht="18.75">
+    <row r="218" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A218" s="1">
         <v>6055000013</v>
       </c>
@@ -3914,7 +3907,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="219" spans="1:3" ht="18.75">
+    <row r="219" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A219" s="1">
         <v>6056000000</v>
       </c>
@@ -3925,7 +3918,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="220" spans="1:3" ht="18.75">
+    <row r="220" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A220" s="1">
         <v>6056000001</v>
       </c>
@@ -3936,7 +3929,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="221" spans="1:3" ht="18.75">
+    <row r="221" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A221" s="1">
         <v>6056000002</v>
       </c>
@@ -3947,7 +3940,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="222" spans="1:3" ht="18.75">
+    <row r="222" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A222" s="1">
         <v>6056000003</v>
       </c>
@@ -3958,7 +3951,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="223" spans="1:3" ht="18.75">
+    <row r="223" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A223" s="1">
         <v>6056000004</v>
       </c>
@@ -3969,7 +3962,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="224" spans="1:3" ht="18.75">
+    <row r="224" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A224" s="1">
         <v>6056000005</v>
       </c>
@@ -3980,7 +3973,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="225" spans="1:3" ht="18.75">
+    <row r="225" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A225" s="1">
         <v>6056000006</v>
       </c>
@@ -3991,7 +3984,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="226" spans="1:3" ht="18.75">
+    <row r="226" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A226" s="1">
         <v>6056000007</v>
       </c>
@@ -4002,7 +3995,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="227" spans="1:3" ht="18.75">
+    <row r="227" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A227" s="1">
         <v>6056000008</v>
       </c>
@@ -4013,7 +4006,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="228" spans="1:3" ht="18.75">
+    <row r="228" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A228" s="1">
         <v>6056000009</v>
       </c>
@@ -4024,7 +4017,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="229" spans="1:3" ht="18.75">
+    <row r="229" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A229" s="1">
         <v>6056000010</v>
       </c>
@@ -4035,7 +4028,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="230" spans="1:3" ht="18.75">
+    <row r="230" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A230" s="1">
         <v>6056000011</v>
       </c>
@@ -4046,7 +4039,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="231" spans="1:3" ht="18.75">
+    <row r="231" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A231" s="1">
         <v>6056000012</v>
       </c>
@@ -4057,7 +4050,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="232" spans="1:3" ht="18.75">
+    <row r="232" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A232" s="1">
         <v>6056000013</v>
       </c>
@@ -4068,7 +4061,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="233" spans="1:3" ht="18.75">
+    <row r="233" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A233" s="1">
         <v>6056000014</v>
       </c>
@@ -4079,7 +4072,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="234" spans="1:3" ht="18.75">
+    <row r="234" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A234" s="1">
         <v>6056000015</v>
       </c>
@@ -4090,7 +4083,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="235" spans="1:3" ht="18.75">
+    <row r="235" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A235" s="1">
         <v>6056000016</v>
       </c>
@@ -4101,7 +4094,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="236" spans="1:3" ht="18.75">
+    <row r="236" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A236" s="1">
         <v>6056000017</v>
       </c>
@@ -4112,7 +4105,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="237" spans="1:3" ht="18.75">
+    <row r="237" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A237" s="1">
         <v>6056000018</v>
       </c>
@@ -4123,7 +4116,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="238" spans="1:3" ht="18.75">
+    <row r="238" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A238" s="1">
         <v>6056000019</v>
       </c>
@@ -4134,7 +4127,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="239" spans="1:3" ht="18.75">
+    <row r="239" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A239" s="1">
         <v>6056000020</v>
       </c>
@@ -4145,7 +4138,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="240" spans="1:3" ht="18.75">
+    <row r="240" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A240" s="1">
         <v>6056000021</v>
       </c>
@@ -4156,7 +4149,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="241" spans="1:3" ht="18.75">
+    <row r="241" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A241" s="1">
         <v>6056000022</v>
       </c>
@@ -4167,7 +4160,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="242" spans="1:3" ht="18.75">
+    <row r="242" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A242" s="1">
         <v>6056000023</v>
       </c>
@@ -4178,7 +4171,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="243" spans="1:3" ht="18.75">
+    <row r="243" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A243" s="1">
         <v>6056000024</v>
       </c>
@@ -4189,7 +4182,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="244" spans="1:3" ht="18.75">
+    <row r="244" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A244" s="1">
         <v>6056000025</v>
       </c>
@@ -4200,7 +4193,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="245" spans="1:3" ht="18.75">
+    <row r="245" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A245" s="1">
         <v>6056000026</v>
       </c>
@@ -4211,7 +4204,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="246" spans="1:3" ht="18.75">
+    <row r="246" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A246" s="1">
         <v>6056000027</v>
       </c>
@@ -4222,7 +4215,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="247" spans="1:3" ht="18.75">
+    <row r="247" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A247" s="1">
         <v>6056000028</v>
       </c>
@@ -4233,7 +4226,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="248" spans="1:3" ht="18.75">
+    <row r="248" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A248" s="1">
         <v>6056000029</v>
       </c>
@@ -4244,7 +4237,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="249" spans="1:3" ht="18.75">
+    <row r="249" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A249" s="1">
         <v>6056000030</v>
       </c>
@@ -4255,7 +4248,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="250" spans="1:3" ht="18.75">
+    <row r="250" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A250" s="1">
         <v>6056000031</v>
       </c>
@@ -4266,7 +4259,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="251" spans="1:3" ht="18.75">
+    <row r="251" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A251" s="1">
         <v>6056000032</v>
       </c>
@@ -4277,7 +4270,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="252" spans="1:3" ht="18.75">
+    <row r="252" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A252" s="1">
         <v>6056000033</v>
       </c>
@@ -4288,7 +4281,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="253" spans="1:3" ht="18.75">
+    <row r="253" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A253" s="1">
         <v>6056000034</v>
       </c>
@@ -4299,7 +4292,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="254" spans="1:3" ht="18.75">
+    <row r="254" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A254" s="1">
         <v>6056000035</v>
       </c>
@@ -4310,7 +4303,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="255" spans="1:3" ht="18.75">
+    <row r="255" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A255" s="1">
         <v>6056000036</v>
       </c>
@@ -4321,7 +4314,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="256" spans="1:3" ht="18.75">
+    <row r="256" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A256" s="1">
         <v>6056000037</v>
       </c>
@@ -4332,7 +4325,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="257" spans="1:3" ht="18.75">
+    <row r="257" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A257" s="1">
         <v>6056000038</v>
       </c>
@@ -4343,7 +4336,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="258" spans="1:3" ht="18.75">
+    <row r="258" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A258" s="1">
         <v>6056000039</v>
       </c>
@@ -4354,7 +4347,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="259" spans="1:3" ht="18.75">
+    <row r="259" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A259" s="1">
         <v>6056000040</v>
       </c>
@@ -4365,7 +4358,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="260" spans="1:3" ht="18.75">
+    <row r="260" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A260" s="1">
         <v>6056000041</v>
       </c>
@@ -4376,7 +4369,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="261" spans="1:3" ht="18.75">
+    <row r="261" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A261" s="1">
         <v>6056000042</v>
       </c>
@@ -4387,7 +4380,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="262" spans="1:3" ht="18.75">
+    <row r="262" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A262" s="1">
         <v>6056000043</v>
       </c>
@@ -4398,7 +4391,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="263" spans="1:3" ht="18.75">
+    <row r="263" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A263" s="1">
         <v>6056000044</v>
       </c>
@@ -4409,7 +4402,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="264" spans="1:3" ht="18.75">
+    <row r="264" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A264" s="1">
         <v>6056000045</v>
       </c>
@@ -4420,7 +4413,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="265" spans="1:3" ht="18.75">
+    <row r="265" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A265" s="1">
         <v>6056000046</v>
       </c>
@@ -4431,7 +4424,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="266" spans="1:3" ht="18.75">
+    <row r="266" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A266" s="1">
         <v>6056000047</v>
       </c>
@@ -4442,7 +4435,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="267" spans="1:3" ht="18.75">
+    <row r="267" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A267" s="1">
         <v>6056000048</v>
       </c>
@@ -4453,7 +4446,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="268" spans="1:3" ht="18.75">
+    <row r="268" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A268" s="1">
         <v>6056000049</v>
       </c>
@@ -4464,7 +4457,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="269" spans="1:3" ht="18.75">
+    <row r="269" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A269" s="1">
         <v>6056000050</v>
       </c>
@@ -4475,7 +4468,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="270" spans="1:3" ht="18.75">
+    <row r="270" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A270" s="1">
         <v>6056000051</v>
       </c>
@@ -4486,7 +4479,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="271" spans="1:3" ht="18.75">
+    <row r="271" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A271" s="1">
         <v>6056000052</v>
       </c>
@@ -4497,7 +4490,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="272" spans="1:3" ht="18.75">
+    <row r="272" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A272" s="1">
         <v>6056000053</v>
       </c>
@@ -4508,7 +4501,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="273" spans="1:3" ht="18.75">
+    <row r="273" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A273" s="1">
         <v>6056000054</v>
       </c>
@@ -4519,7 +4512,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="274" spans="1:3" ht="18.75">
+    <row r="274" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A274" s="1">
         <v>6056000055</v>
       </c>
@@ -4530,7 +4523,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="275" spans="1:3" ht="18.75">
+    <row r="275" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A275" s="1">
         <v>6056000056</v>
       </c>
@@ -4541,7 +4534,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="276" spans="1:3" ht="18.75">
+    <row r="276" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A276" s="1">
         <v>6056000057</v>
       </c>
@@ -4552,7 +4545,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="277" spans="1:3" ht="18.75">
+    <row r="277" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A277" s="1">
         <v>6056000058</v>
       </c>
@@ -4563,7 +4556,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="278" spans="1:3" ht="18.75">
+    <row r="278" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A278" s="1">
         <v>6056000059</v>
       </c>
@@ -4574,7 +4567,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="279" spans="1:3" ht="18.75">
+    <row r="279" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A279" s="1">
         <v>6080000001</v>
       </c>
@@ -4585,7 +4578,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="280" spans="1:3" ht="18.75">
+    <row r="280" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A280" s="1">
         <v>6080000002</v>
       </c>
@@ -4596,7 +4589,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="281" spans="1:3" ht="18.75">
+    <row r="281" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A281" s="1">
         <v>6080000003</v>
       </c>
@@ -4607,7 +4600,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="282" spans="1:3" ht="18.75">
+    <row r="282" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A282" s="1">
         <v>6080000004</v>
       </c>
@@ -4618,7 +4611,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="283" spans="1:3" ht="18.75">
+    <row r="283" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A283" s="1">
         <v>6080000005</v>
       </c>
@@ -4629,7 +4622,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="284" spans="1:3" ht="18.75">
+    <row r="284" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A284" s="2">
         <v>6140000000</v>
       </c>
@@ -4640,7 +4633,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="285" spans="1:3" ht="18.75">
+    <row r="285" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A285" s="1">
         <v>6220000000</v>
       </c>
@@ -4651,7 +4644,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="286" spans="1:3" ht="18.75">
+    <row r="286" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A286" s="1">
         <v>6223000001</v>
       </c>
@@ -4662,7 +4655,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="287" spans="1:3" ht="18.75">
+    <row r="287" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A287" s="1">
         <v>6223000002</v>
       </c>
@@ -4673,7 +4666,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="288" spans="1:3" ht="18.75">
+    <row r="288" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A288" s="1">
         <v>6223000003</v>
       </c>
@@ -4684,7 +4677,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="289" spans="1:3" ht="18.75">
+    <row r="289" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A289" s="1">
         <v>6223000004</v>
       </c>
@@ -4695,7 +4688,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="290" spans="1:3" ht="18.75">
+    <row r="290" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A290" s="1">
         <v>6223000005</v>
       </c>
@@ -4706,7 +4699,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="291" spans="1:3" ht="18.75">
+    <row r="291" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A291" s="1">
         <v>6223000006</v>
       </c>
@@ -4717,7 +4710,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="292" spans="1:3" ht="18.75">
+    <row r="292" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A292" s="1">
         <v>6223000007</v>
       </c>
@@ -4728,7 +4721,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="293" spans="1:3" ht="18.75">
+    <row r="293" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A293" s="1">
         <v>6223000008</v>
       </c>
@@ -4739,7 +4732,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="294" spans="1:3" ht="18.75">
+    <row r="294" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A294" s="1">
         <v>6223000009</v>
       </c>
@@ -4750,7 +4743,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="295" spans="1:3" ht="18.75">
+    <row r="295" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A295" s="1">
         <v>6240000000</v>
       </c>
@@ -4761,7 +4754,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="296" spans="1:3" ht="18.75">
+    <row r="296" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A296" s="1">
         <v>6240000001</v>
       </c>
@@ -4772,7 +4765,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="297" spans="1:3" ht="18.75">
+    <row r="297" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A297" s="1">
         <v>6240000002</v>
       </c>
@@ -4783,7 +4776,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="298" spans="1:3" ht="18.75">
+    <row r="298" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A298" s="1">
         <v>6240000003</v>
       </c>
@@ -4794,7 +4787,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="299" spans="1:3" ht="18.75">
+    <row r="299" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A299" s="1">
         <v>6240000004</v>
       </c>
@@ -4805,7 +4798,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="300" spans="1:3" ht="18.75">
+    <row r="300" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A300" s="1">
         <v>6240000005</v>
       </c>
@@ -4816,7 +4809,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="301" spans="1:3" ht="18.75">
+    <row r="301" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A301" s="1">
         <v>6240000006</v>
       </c>
@@ -4827,7 +4820,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="302" spans="1:3" ht="18.75">
+    <row r="302" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A302" s="1">
         <v>6240000007</v>
       </c>
@@ -4838,7 +4831,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="303" spans="1:3" ht="18.75">
+    <row r="303" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A303" s="1">
         <v>6240000008</v>
       </c>
@@ -4849,7 +4842,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="304" spans="1:3" ht="18.75">
+    <row r="304" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A304" s="1">
         <v>6240000009</v>
       </c>
@@ -4860,7 +4853,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="305" spans="1:3" ht="18.75">
+    <row r="305" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A305" s="1">
         <v>6288000000</v>
       </c>
@@ -4871,7 +4864,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="306" spans="1:3" ht="18.75">
+    <row r="306" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A306" s="1">
         <v>6384000001</v>
       </c>
@@ -4882,7 +4875,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="307" spans="1:3" ht="18.75">
+    <row r="307" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A307" s="1">
         <v>6384000002</v>
       </c>
@@ -4893,7 +4886,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="308" spans="1:3" ht="18.75">
+    <row r="308" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A308" s="1">
         <v>6500000000</v>
       </c>
@@ -4904,7 +4897,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="309" spans="1:3" ht="18.75">
+    <row r="309" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A309" s="1">
         <v>6620000000</v>
       </c>
@@ -4915,7 +4908,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="310" spans="1:3" ht="18.75">
+    <row r="310" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A310" s="1">
         <v>6631000000</v>
       </c>
@@ -4926,7 +4919,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="311" spans="1:3" ht="18.75">
+    <row r="311" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A311" s="1">
         <v>6672000000</v>
       </c>
@@ -4937,7 +4930,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="312" spans="1:3" ht="18.75">
+    <row r="312" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A312" s="1">
         <v>6672000001</v>
       </c>
@@ -4948,7 +4941,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="313" spans="1:3" ht="18.75">
+    <row r="313" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A313" s="1">
         <v>6672000002</v>
       </c>
@@ -4959,7 +4952,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="314" spans="1:3" ht="18.75">
+    <row r="314" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A314" s="1">
         <v>6672000003</v>
       </c>
@@ -4970,7 +4963,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="315" spans="1:3" ht="18.75">
+    <row r="315" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A315" s="1">
         <v>6730000000</v>
       </c>
@@ -4981,7 +4974,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="316" spans="1:3" ht="18.75">
+    <row r="316" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A316" s="1">
         <v>6760000000</v>
       </c>
@@ -4992,7 +4985,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="317" spans="1:3" ht="18.75">
+    <row r="317" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A317" s="1">
         <v>6810000000</v>
       </c>
@@ -5003,7 +4996,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="318" spans="1:3" ht="18.75">
+    <row r="318" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A318" s="1">
         <v>7010000001</v>
       </c>
@@ -5014,7 +5007,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="319" spans="1:3" ht="18.75">
+    <row r="319" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A319" s="1">
         <v>7010000002</v>
       </c>
@@ -5025,7 +5018,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="320" spans="1:3" ht="18.75">
+    <row r="320" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A320" s="1">
         <v>7010000003</v>
       </c>
@@ -5036,7 +5029,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="321" spans="1:3" ht="18.75">
+    <row r="321" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A321" s="1">
         <v>7010000004</v>
       </c>
@@ -5047,7 +5040,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="322" spans="1:3" ht="18.75">
+    <row r="322" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A322" s="1">
         <v>7010000005</v>
       </c>
@@ -5058,7 +5051,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="323" spans="1:3" ht="18.75">
+    <row r="323" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A323" s="1">
         <v>7010000006</v>
       </c>
@@ -5069,7 +5062,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="324" spans="1:3" ht="18.75">
+    <row r="324" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A324" s="1">
         <v>7010000007</v>
       </c>
@@ -5080,7 +5073,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="325" spans="1:3" ht="18.75">
+    <row r="325" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A325" s="1">
         <v>7010000008</v>
       </c>
@@ -5091,7 +5084,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="326" spans="1:3" ht="18.75">
+    <row r="326" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A326" s="1">
         <v>7010000009</v>
       </c>
@@ -5102,7 +5095,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="327" spans="1:3" ht="18.75">
+    <row r="327" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A327" s="1">
         <v>7010000010</v>
       </c>
@@ -5113,7 +5106,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="328" spans="1:3" ht="18.75">
+    <row r="328" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A328" s="1">
         <v>7010000011</v>
       </c>
@@ -5124,7 +5117,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="329" spans="1:3" ht="18.75">
+    <row r="329" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A329" s="1">
         <v>7010000012</v>
       </c>
@@ -5135,7 +5128,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="330" spans="1:3" ht="18.75">
+    <row r="330" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A330" s="1">
         <v>7060000000</v>
       </c>
@@ -5146,7 +5139,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="331" spans="1:3" ht="18.75">
+    <row r="331" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A331" s="1">
         <v>7588000000</v>
       </c>
@@ -5157,7 +5150,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="332" spans="1:3" ht="18.75">
+    <row r="332" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A332" s="1">
         <v>7760000000</v>
       </c>
@@ -5168,7 +5161,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="333" spans="1:3" ht="18.75">
+    <row r="333" spans="1:3" ht="18" x14ac:dyDescent="0.4">
       <c r="A333" s="1">
         <v>7870000000</v>
       </c>
@@ -5177,6 +5170,17 @@
       </c>
       <c r="C333" s="1" t="s">
         <v>322</v>
+      </c>
+    </row>
+    <row r="334" spans="1:3" ht="18" x14ac:dyDescent="0.4">
+      <c r="A334" s="8">
+        <v>8910000000</v>
+      </c>
+      <c r="B334" s="8" t="s">
+        <v>338</v>
+      </c>
+      <c r="C334" s="8" t="s">
+        <v>157</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
non affichage du compte 4211 au bilan
</commit_message>
<xml_diff>
--- a/public/PLAN.xlsx
+++ b/public/PLAN.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="667" uniqueCount="342">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="675" uniqueCount="346">
   <si>
     <t>Comptes</t>
   </si>
@@ -179,6 +179,12 @@
     <t>Land cruser</t>
   </si>
   <si>
+    <t>Sarf</t>
+  </si>
+  <si>
+    <t>Appareil topographique</t>
+  </si>
+  <si>
     <t>Amortissement starling</t>
   </si>
   <si>
@@ -273,6 +279,12 @@
   </si>
   <si>
     <t>Amortissement batiment</t>
+  </si>
+  <si>
+    <t>Amortissement Sarf</t>
+  </si>
+  <si>
+    <t>Amortissement Appareil topographique</t>
   </si>
   <si>
     <t>Salopettes</t>
@@ -1066,7 +1078,7 @@
     <numFmt numFmtId="177" formatCode="_-&quot;€&quot;* #,##0_-;\-&quot;€&quot;* #,##0_-;_-&quot;€&quot;* \-_-;_-@_-"/>
     <numFmt numFmtId="178" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1086,13 +1098,6 @@
       <color theme="1"/>
       <name val="Times New Roman"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -1254,7 +1259,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1447,12 +1452,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="12">
     <border>
@@ -1602,28 +1601,31 @@
   </borders>
   <cellStyleXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1632,125 +1634,122 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="33" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -2121,7 +2120,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C337"/>
+  <dimension ref="A1:C341"/>
   <sheetFormatPr defaultColWidth="11.4571428571429" defaultRowHeight="15" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="19.4571428571429" customWidth="1"/>
@@ -2634,7 +2633,7 @@
     </row>
     <row r="48" ht="18.75" spans="1:3">
       <c r="A48" s="2">
-        <v>2810000001</v>
+        <v>2451000005</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>50</v>
@@ -2645,7 +2644,7 @@
     </row>
     <row r="49" ht="18.75" spans="1:3">
       <c r="A49" s="2">
-        <v>2810000002</v>
+        <v>2480000001</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>51</v>
@@ -2656,7 +2655,7 @@
     </row>
     <row r="50" ht="18.75" spans="1:3">
       <c r="A50" s="2">
-        <v>2810000003</v>
+        <v>2810000001</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>52</v>
@@ -2667,7 +2666,7 @@
     </row>
     <row r="51" ht="18.75" spans="1:3">
       <c r="A51" s="2">
-        <v>2810000004</v>
+        <v>2810000002</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>53</v>
@@ -2678,7 +2677,7 @@
     </row>
     <row r="52" ht="18.75" spans="1:3">
       <c r="A52" s="2">
-        <v>2840000001</v>
+        <v>2810000003</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>54</v>
@@ -2689,7 +2688,7 @@
     </row>
     <row r="53" ht="18.75" spans="1:3">
       <c r="A53" s="2">
-        <v>2840000002</v>
+        <v>2810000004</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>55</v>
@@ -2700,7 +2699,7 @@
     </row>
     <row r="54" ht="18.75" spans="1:3">
       <c r="A54" s="2">
-        <v>2840000003</v>
+        <v>2840000001</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>56</v>
@@ -2711,7 +2710,7 @@
     </row>
     <row r="55" ht="18.75" spans="1:3">
       <c r="A55" s="2">
-        <v>2840000004</v>
+        <v>2840000002</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>57</v>
@@ -2722,7 +2721,7 @@
     </row>
     <row r="56" ht="18.75" spans="1:3">
       <c r="A56" s="2">
-        <v>2840000005</v>
+        <v>2840000003</v>
       </c>
       <c r="B56" s="2" t="s">
         <v>58</v>
@@ -2733,7 +2732,7 @@
     </row>
     <row r="57" ht="18.75" spans="1:3">
       <c r="A57" s="2">
-        <v>2840000006</v>
+        <v>2840000004</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>59</v>
@@ -2744,7 +2743,7 @@
     </row>
     <row r="58" ht="18.75" spans="1:3">
       <c r="A58" s="2">
-        <v>2840000007</v>
+        <v>2840000005</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>60</v>
@@ -2755,7 +2754,7 @@
     </row>
     <row r="59" ht="18.75" spans="1:3">
       <c r="A59" s="2">
-        <v>2840000008</v>
+        <v>2840000006</v>
       </c>
       <c r="B59" s="2" t="s">
         <v>61</v>
@@ -2766,7 +2765,7 @@
     </row>
     <row r="60" ht="18.75" spans="1:3">
       <c r="A60" s="2">
-        <v>2840000009</v>
+        <v>2840000007</v>
       </c>
       <c r="B60" s="2" t="s">
         <v>62</v>
@@ -2777,7 +2776,7 @@
     </row>
     <row r="61" ht="18.75" spans="1:3">
       <c r="A61" s="2">
-        <v>2840000010</v>
+        <v>2840000008</v>
       </c>
       <c r="B61" s="2" t="s">
         <v>63</v>
@@ -2788,7 +2787,7 @@
     </row>
     <row r="62" ht="18.75" spans="1:3">
       <c r="A62" s="2">
-        <v>2840000011</v>
+        <v>2840000009</v>
       </c>
       <c r="B62" s="2" t="s">
         <v>64</v>
@@ -2799,7 +2798,7 @@
     </row>
     <row r="63" ht="18.75" spans="1:3">
       <c r="A63" s="2">
-        <v>2840000012</v>
+        <v>2840000010</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>65</v>
@@ -2810,7 +2809,7 @@
     </row>
     <row r="64" ht="18.75" spans="1:3">
       <c r="A64" s="2">
-        <v>2840000013</v>
+        <v>2840000011</v>
       </c>
       <c r="B64" s="2" t="s">
         <v>66</v>
@@ -2821,7 +2820,7 @@
     </row>
     <row r="65" ht="18.75" spans="1:3">
       <c r="A65" s="2">
-        <v>2840000014</v>
+        <v>2840000012</v>
       </c>
       <c r="B65" s="2" t="s">
         <v>67</v>
@@ -2832,7 +2831,7 @@
     </row>
     <row r="66" ht="18.75" spans="1:3">
       <c r="A66" s="2">
-        <v>2840000015</v>
+        <v>2840000013</v>
       </c>
       <c r="B66" s="2" t="s">
         <v>68</v>
@@ -2843,7 +2842,7 @@
     </row>
     <row r="67" ht="18.75" spans="1:3">
       <c r="A67" s="2">
-        <v>2840000016</v>
+        <v>2840000014</v>
       </c>
       <c r="B67" s="2" t="s">
         <v>69</v>
@@ -2854,7 +2853,7 @@
     </row>
     <row r="68" ht="18.75" spans="1:3">
       <c r="A68" s="2">
-        <v>2840000017</v>
+        <v>2840000015</v>
       </c>
       <c r="B68" s="2" t="s">
         <v>70</v>
@@ -2865,7 +2864,7 @@
     </row>
     <row r="69" ht="18.75" spans="1:3">
       <c r="A69" s="2">
-        <v>2840000018</v>
+        <v>2840000016</v>
       </c>
       <c r="B69" s="2" t="s">
         <v>71</v>
@@ -2876,7 +2875,7 @@
     </row>
     <row r="70" ht="18.75" spans="1:3">
       <c r="A70" s="2">
-        <v>2840000019</v>
+        <v>2840000017</v>
       </c>
       <c r="B70" s="2" t="s">
         <v>72</v>
@@ -2887,7 +2886,7 @@
     </row>
     <row r="71" ht="18.75" spans="1:3">
       <c r="A71" s="2">
-        <v>2840000020</v>
+        <v>2840000018</v>
       </c>
       <c r="B71" s="2" t="s">
         <v>73</v>
@@ -2898,7 +2897,7 @@
     </row>
     <row r="72" ht="18.75" spans="1:3">
       <c r="A72" s="2">
-        <v>2840000021</v>
+        <v>2840000019</v>
       </c>
       <c r="B72" s="2" t="s">
         <v>74</v>
@@ -2909,7 +2908,7 @@
     </row>
     <row r="73" ht="18.75" spans="1:3">
       <c r="A73" s="2">
-        <v>2840000022</v>
+        <v>2840000020</v>
       </c>
       <c r="B73" s="2" t="s">
         <v>75</v>
@@ -2920,7 +2919,7 @@
     </row>
     <row r="74" ht="18.75" spans="1:3">
       <c r="A74" s="2">
-        <v>2840000023</v>
+        <v>2840000021</v>
       </c>
       <c r="B74" s="2" t="s">
         <v>76</v>
@@ -2931,7 +2930,7 @@
     </row>
     <row r="75" ht="18.75" spans="1:3">
       <c r="A75" s="2">
-        <v>2840000024</v>
+        <v>2840000022</v>
       </c>
       <c r="B75" s="2" t="s">
         <v>77</v>
@@ -2942,7 +2941,7 @@
     </row>
     <row r="76" ht="18.75" spans="1:3">
       <c r="A76" s="2">
-        <v>2840000025</v>
+        <v>2840000023</v>
       </c>
       <c r="B76" s="2" t="s">
         <v>78</v>
@@ -2953,7 +2952,7 @@
     </row>
     <row r="77" ht="18.75" spans="1:3">
       <c r="A77" s="2">
-        <v>2840000026</v>
+        <v>2840000024</v>
       </c>
       <c r="B77" s="2" t="s">
         <v>79</v>
@@ -2964,7 +2963,7 @@
     </row>
     <row r="78" ht="18.75" spans="1:3">
       <c r="A78" s="2">
-        <v>2840000027</v>
+        <v>2840000025</v>
       </c>
       <c r="B78" s="2" t="s">
         <v>80</v>
@@ -2975,7 +2974,7 @@
     </row>
     <row r="79" ht="18.75" spans="1:3">
       <c r="A79" s="2">
-        <v>2840000028</v>
+        <v>2840000026</v>
       </c>
       <c r="B79" s="2" t="s">
         <v>81</v>
@@ -2986,7 +2985,7 @@
     </row>
     <row r="80" ht="18.75" spans="1:3">
       <c r="A80" s="2">
-        <v>3340000001</v>
+        <v>2840000027</v>
       </c>
       <c r="B80" s="2" t="s">
         <v>82</v>
@@ -2997,7 +2996,7 @@
     </row>
     <row r="81" ht="18.75" spans="1:3">
       <c r="A81" s="2">
-        <v>3340000002</v>
+        <v>2840000028</v>
       </c>
       <c r="B81" s="2" t="s">
         <v>83</v>
@@ -3008,7 +3007,7 @@
     </row>
     <row r="82" ht="18.75" spans="1:3">
       <c r="A82" s="2">
-        <v>3340000003</v>
+        <v>2840000029</v>
       </c>
       <c r="B82" s="2" t="s">
         <v>84</v>
@@ -3019,7 +3018,7 @@
     </row>
     <row r="83" ht="18.75" spans="1:3">
       <c r="A83" s="2">
-        <v>3340000004</v>
+        <v>2840000030</v>
       </c>
       <c r="B83" s="2" t="s">
         <v>85</v>
@@ -3030,7 +3029,7 @@
     </row>
     <row r="84" ht="18.75" spans="1:3">
       <c r="A84" s="2">
-        <v>3340000005</v>
+        <v>3340000001</v>
       </c>
       <c r="B84" s="2" t="s">
         <v>86</v>
@@ -3041,7 +3040,7 @@
     </row>
     <row r="85" ht="18.75" spans="1:3">
       <c r="A85" s="2">
-        <v>3340000006</v>
+        <v>3340000002</v>
       </c>
       <c r="B85" s="2" t="s">
         <v>87</v>
@@ -3052,7 +3051,7 @@
     </row>
     <row r="86" ht="18.75" spans="1:3">
       <c r="A86" s="2">
-        <v>3340000007</v>
+        <v>3340000003</v>
       </c>
       <c r="B86" s="2" t="s">
         <v>88</v>
@@ -3063,7 +3062,7 @@
     </row>
     <row r="87" ht="18.75" spans="1:3">
       <c r="A87" s="2">
-        <v>3340000008</v>
+        <v>3340000004</v>
       </c>
       <c r="B87" s="2" t="s">
         <v>89</v>
@@ -3074,7 +3073,7 @@
     </row>
     <row r="88" ht="18.75" spans="1:3">
       <c r="A88" s="2">
-        <v>3340000009</v>
+        <v>3340000005</v>
       </c>
       <c r="B88" s="2" t="s">
         <v>90</v>
@@ -3085,7 +3084,7 @@
     </row>
     <row r="89" ht="18.75" spans="1:3">
       <c r="A89" s="2">
-        <v>3340000010</v>
+        <v>3340000006</v>
       </c>
       <c r="B89" s="2" t="s">
         <v>91</v>
@@ -3096,7 +3095,7 @@
     </row>
     <row r="90" ht="18.75" spans="1:3">
       <c r="A90" s="2">
-        <v>3340000011</v>
+        <v>3340000007</v>
       </c>
       <c r="B90" s="2" t="s">
         <v>92</v>
@@ -3107,7 +3106,7 @@
     </row>
     <row r="91" ht="18.75" spans="1:3">
       <c r="A91" s="2">
-        <v>3340000012</v>
+        <v>3340000008</v>
       </c>
       <c r="B91" s="2" t="s">
         <v>93</v>
@@ -3118,7 +3117,7 @@
     </row>
     <row r="92" ht="18.75" spans="1:3">
       <c r="A92" s="2">
-        <v>3340000013</v>
+        <v>3340000009</v>
       </c>
       <c r="B92" s="2" t="s">
         <v>94</v>
@@ -3129,7 +3128,7 @@
     </row>
     <row r="93" ht="18.75" spans="1:3">
       <c r="A93" s="2">
-        <v>3340000014</v>
+        <v>3340000010</v>
       </c>
       <c r="B93" s="2" t="s">
         <v>95</v>
@@ -3140,7 +3139,7 @@
     </row>
     <row r="94" ht="18.75" spans="1:3">
       <c r="A94" s="2">
-        <v>3340000015</v>
+        <v>3340000011</v>
       </c>
       <c r="B94" s="2" t="s">
         <v>96</v>
@@ -3151,7 +3150,7 @@
     </row>
     <row r="95" ht="18.75" spans="1:3">
       <c r="A95" s="2">
-        <v>3340000016</v>
+        <v>3340000012</v>
       </c>
       <c r="B95" s="2" t="s">
         <v>97</v>
@@ -3162,7 +3161,7 @@
     </row>
     <row r="96" ht="18.75" spans="1:3">
       <c r="A96" s="2">
-        <v>3340000017</v>
+        <v>3340000013</v>
       </c>
       <c r="B96" s="2" t="s">
         <v>98</v>
@@ -3173,7 +3172,7 @@
     </row>
     <row r="97" ht="18.75" spans="1:3">
       <c r="A97" s="2">
-        <v>3340000018</v>
+        <v>3340000014</v>
       </c>
       <c r="B97" s="2" t="s">
         <v>99</v>
@@ -3184,7 +3183,7 @@
     </row>
     <row r="98" ht="18.75" spans="1:3">
       <c r="A98" s="2">
-        <v>3340000019</v>
+        <v>3340000015</v>
       </c>
       <c r="B98" s="2" t="s">
         <v>100</v>
@@ -3195,7 +3194,7 @@
     </row>
     <row r="99" ht="18.75" spans="1:3">
       <c r="A99" s="2">
-        <v>3340000020</v>
+        <v>3340000016</v>
       </c>
       <c r="B99" s="2" t="s">
         <v>101</v>
@@ -3206,7 +3205,7 @@
     </row>
     <row r="100" ht="18.75" spans="1:3">
       <c r="A100" s="2">
-        <v>3340000021</v>
+        <v>3340000017</v>
       </c>
       <c r="B100" s="2" t="s">
         <v>102</v>
@@ -3217,7 +3216,7 @@
     </row>
     <row r="101" ht="18.75" spans="1:3">
       <c r="A101" s="2">
-        <v>3340000022</v>
+        <v>3340000018</v>
       </c>
       <c r="B101" s="2" t="s">
         <v>103</v>
@@ -3228,7 +3227,7 @@
     </row>
     <row r="102" ht="18.75" spans="1:3">
       <c r="A102" s="2">
-        <v>3340000023</v>
+        <v>3340000019</v>
       </c>
       <c r="B102" s="2" t="s">
         <v>104</v>
@@ -3239,7 +3238,7 @@
     </row>
     <row r="103" ht="18.75" spans="1:3">
       <c r="A103" s="2">
-        <v>3340000024</v>
+        <v>3340000020</v>
       </c>
       <c r="B103" s="2" t="s">
         <v>105</v>
@@ -3250,7 +3249,7 @@
     </row>
     <row r="104" ht="18.75" spans="1:3">
       <c r="A104" s="2">
-        <v>3340000025</v>
+        <v>3340000021</v>
       </c>
       <c r="B104" s="2" t="s">
         <v>106</v>
@@ -3261,7 +3260,7 @@
     </row>
     <row r="105" ht="18.75" spans="1:3">
       <c r="A105" s="2">
-        <v>3340000026</v>
+        <v>3340000022</v>
       </c>
       <c r="B105" s="2" t="s">
         <v>107</v>
@@ -3272,7 +3271,7 @@
     </row>
     <row r="106" ht="18.75" spans="1:3">
       <c r="A106" s="2">
-        <v>3340000027</v>
+        <v>3340000023</v>
       </c>
       <c r="B106" s="2" t="s">
         <v>108</v>
@@ -3283,7 +3282,7 @@
     </row>
     <row r="107" ht="18.75" spans="1:3">
       <c r="A107" s="2">
-        <v>3340000028</v>
+        <v>3340000024</v>
       </c>
       <c r="B107" s="2" t="s">
         <v>109</v>
@@ -3294,7 +3293,7 @@
     </row>
     <row r="108" ht="18.75" spans="1:3">
       <c r="A108" s="2">
-        <v>3340000029</v>
+        <v>3340000025</v>
       </c>
       <c r="B108" s="2" t="s">
         <v>110</v>
@@ -3305,7 +3304,7 @@
     </row>
     <row r="109" ht="18.75" spans="1:3">
       <c r="A109" s="2">
-        <v>3340000030</v>
+        <v>3340000026</v>
       </c>
       <c r="B109" s="2" t="s">
         <v>111</v>
@@ -3316,7 +3315,7 @@
     </row>
     <row r="110" ht="18.75" spans="1:3">
       <c r="A110" s="2">
-        <v>3340000031</v>
+        <v>3340000027</v>
       </c>
       <c r="B110" s="2" t="s">
         <v>112</v>
@@ -3327,7 +3326,7 @@
     </row>
     <row r="111" ht="18.75" spans="1:3">
       <c r="A111" s="2">
-        <v>3340000032</v>
+        <v>3340000028</v>
       </c>
       <c r="B111" s="2" t="s">
         <v>113</v>
@@ -3338,7 +3337,7 @@
     </row>
     <row r="112" ht="18.75" spans="1:3">
       <c r="A112" s="2">
-        <v>3340000033</v>
+        <v>3340000029</v>
       </c>
       <c r="B112" s="2" t="s">
         <v>114</v>
@@ -3349,7 +3348,7 @@
     </row>
     <row r="113" ht="18.75" spans="1:3">
       <c r="A113" s="2">
-        <v>3340000034</v>
+        <v>3340000030</v>
       </c>
       <c r="B113" s="2" t="s">
         <v>115</v>
@@ -3360,7 +3359,7 @@
     </row>
     <row r="114" ht="18.75" spans="1:3">
       <c r="A114" s="2">
-        <v>3340000035</v>
+        <v>3340000031</v>
       </c>
       <c r="B114" s="2" t="s">
         <v>116</v>
@@ -3371,7 +3370,7 @@
     </row>
     <row r="115" ht="18.75" spans="1:3">
       <c r="A115" s="2">
-        <v>3340000036</v>
+        <v>3340000032</v>
       </c>
       <c r="B115" s="2" t="s">
         <v>117</v>
@@ -3382,7 +3381,7 @@
     </row>
     <row r="116" ht="18.75" spans="1:3">
       <c r="A116" s="2">
-        <v>3340000037</v>
+        <v>3340000033</v>
       </c>
       <c r="B116" s="2" t="s">
         <v>118</v>
@@ -3393,7 +3392,7 @@
     </row>
     <row r="117" ht="18.75" spans="1:3">
       <c r="A117" s="2">
-        <v>3340000038</v>
+        <v>3340000034</v>
       </c>
       <c r="B117" s="2" t="s">
         <v>119</v>
@@ -3404,7 +3403,7 @@
     </row>
     <row r="118" ht="18.75" spans="1:3">
       <c r="A118" s="2">
-        <v>3340000039</v>
+        <v>3340000035</v>
       </c>
       <c r="B118" s="2" t="s">
         <v>120</v>
@@ -3414,8 +3413,8 @@
       </c>
     </row>
     <row r="119" ht="18.75" spans="1:3">
-      <c r="A119" s="3">
-        <v>3340000040</v>
+      <c r="A119" s="2">
+        <v>3340000036</v>
       </c>
       <c r="B119" s="2" t="s">
         <v>121</v>
@@ -3426,7 +3425,7 @@
     </row>
     <row r="120" ht="18.75" spans="1:3">
       <c r="A120" s="2">
-        <v>3340000041</v>
+        <v>3340000037</v>
       </c>
       <c r="B120" s="2" t="s">
         <v>122</v>
@@ -3436,8 +3435,8 @@
       </c>
     </row>
     <row r="121" ht="18.75" spans="1:3">
-      <c r="A121" s="3">
-        <v>3340000042</v>
+      <c r="A121" s="2">
+        <v>3340000038</v>
       </c>
       <c r="B121" s="2" t="s">
         <v>123</v>
@@ -3448,51 +3447,51 @@
     </row>
     <row r="122" ht="18.75" spans="1:3">
       <c r="A122" s="2">
-        <v>4010000001</v>
+        <v>3340000039</v>
       </c>
       <c r="B122" s="2" t="s">
         <v>124</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>3</v>
+        <v>16</v>
       </c>
     </row>
     <row r="123" ht="18.75" spans="1:3">
-      <c r="A123" s="2">
-        <v>4010000021</v>
+      <c r="A123" s="3">
+        <v>3340000040</v>
       </c>
       <c r="B123" s="2" t="s">
         <v>125</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>3</v>
+        <v>16</v>
       </c>
     </row>
     <row r="124" ht="18.75" spans="1:3">
       <c r="A124" s="2">
-        <v>4010000022</v>
+        <v>3340000041</v>
       </c>
       <c r="B124" s="2" t="s">
         <v>126</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>3</v>
+        <v>16</v>
       </c>
     </row>
     <row r="125" ht="18.75" spans="1:3">
-      <c r="A125" s="2">
-        <v>4010000003</v>
+      <c r="A125" s="3">
+        <v>3340000042</v>
       </c>
       <c r="B125" s="2" t="s">
         <v>127</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>3</v>
+        <v>16</v>
       </c>
     </row>
     <row r="126" ht="18.75" spans="1:3">
       <c r="A126" s="2">
-        <v>4010000004</v>
+        <v>4010000001</v>
       </c>
       <c r="B126" s="2" t="s">
         <v>128</v>
@@ -3503,7 +3502,7 @@
     </row>
     <row r="127" ht="18.75" spans="1:3">
       <c r="A127" s="2">
-        <v>4010000005</v>
+        <v>4010000021</v>
       </c>
       <c r="B127" s="2" t="s">
         <v>129</v>
@@ -3514,7 +3513,7 @@
     </row>
     <row r="128" ht="18.75" spans="1:3">
       <c r="A128" s="2">
-        <v>4010000006</v>
+        <v>4010000022</v>
       </c>
       <c r="B128" s="2" t="s">
         <v>130</v>
@@ -3525,7 +3524,7 @@
     </row>
     <row r="129" ht="18.75" spans="1:3">
       <c r="A129" s="2">
-        <v>4010000007</v>
+        <v>4010000003</v>
       </c>
       <c r="B129" s="2" t="s">
         <v>131</v>
@@ -3536,7 +3535,7 @@
     </row>
     <row r="130" ht="18.75" spans="1:3">
       <c r="A130" s="2">
-        <v>4010000008</v>
+        <v>4010000004</v>
       </c>
       <c r="B130" s="2" t="s">
         <v>132</v>
@@ -3547,7 +3546,7 @@
     </row>
     <row r="131" ht="18.75" spans="1:3">
       <c r="A131" s="2">
-        <v>4010000009</v>
+        <v>4010000005</v>
       </c>
       <c r="B131" s="2" t="s">
         <v>133</v>
@@ -3558,7 +3557,7 @@
     </row>
     <row r="132" ht="18.75" spans="1:3">
       <c r="A132" s="2">
-        <v>4010000010</v>
+        <v>4010000006</v>
       </c>
       <c r="B132" s="2" t="s">
         <v>134</v>
@@ -3569,7 +3568,7 @@
     </row>
     <row r="133" ht="18.75" spans="1:3">
       <c r="A133" s="2">
-        <v>4040000000</v>
+        <v>4010000007</v>
       </c>
       <c r="B133" s="2" t="s">
         <v>135</v>
@@ -3580,7 +3579,7 @@
     </row>
     <row r="134" ht="18.75" spans="1:3">
       <c r="A134" s="2">
-        <v>4090000000</v>
+        <v>4010000008</v>
       </c>
       <c r="B134" s="2" t="s">
         <v>136</v>
@@ -3591,18 +3590,18 @@
     </row>
     <row r="135" ht="18.75" spans="1:3">
       <c r="A135" s="2">
-        <v>4110000000</v>
+        <v>4010000009</v>
       </c>
       <c r="B135" s="2" t="s">
         <v>137</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>16</v>
+        <v>3</v>
       </c>
     </row>
     <row r="136" ht="18.75" spans="1:3">
       <c r="A136" s="2">
-        <v>4210000000</v>
+        <v>4010000010</v>
       </c>
       <c r="B136" s="2" t="s">
         <v>138</v>
@@ -3613,7 +3612,7 @@
     </row>
     <row r="137" ht="18.75" spans="1:3">
       <c r="A137" s="2">
-        <v>4211000000</v>
+        <v>4040000000</v>
       </c>
       <c r="B137" s="2" t="s">
         <v>139</v>
@@ -3624,7 +3623,7 @@
     </row>
     <row r="138" ht="18.75" spans="1:3">
       <c r="A138" s="2">
-        <v>4220000000</v>
+        <v>4090000000</v>
       </c>
       <c r="B138" s="2" t="s">
         <v>140</v>
@@ -3635,18 +3634,18 @@
     </row>
     <row r="139" ht="18.75" spans="1:3">
       <c r="A139" s="2">
-        <v>4474000000</v>
+        <v>4110000000</v>
       </c>
       <c r="B139" s="2" t="s">
         <v>141</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>3</v>
+        <v>16</v>
       </c>
     </row>
     <row r="140" ht="18.75" spans="1:3">
       <c r="A140" s="2">
-        <v>4475000000</v>
+        <v>4210000000</v>
       </c>
       <c r="B140" s="2" t="s">
         <v>142</v>
@@ -3657,7 +3656,7 @@
     </row>
     <row r="141" ht="18.75" spans="1:3">
       <c r="A141" s="2">
-        <v>4471000000</v>
+        <v>4211000000</v>
       </c>
       <c r="B141" s="2" t="s">
         <v>143</v>
@@ -3668,7 +3667,7 @@
     </row>
     <row r="142" ht="18.75" spans="1:3">
       <c r="A142" s="2">
-        <v>4472000000</v>
+        <v>4220000000</v>
       </c>
       <c r="B142" s="2" t="s">
         <v>144</v>
@@ -3678,2146 +3677,2190 @@
       </c>
     </row>
     <row r="143" ht="18.75" spans="1:3">
-      <c r="A143" s="5">
-        <v>4620000001</v>
+      <c r="A143" s="2">
+        <v>4474000000</v>
       </c>
       <c r="B143" s="2" t="s">
         <v>145</v>
       </c>
       <c r="C143" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="144" ht="18.75" spans="1:3">
+      <c r="A144" s="2">
+        <v>4475000000</v>
+      </c>
+      <c r="B144" s="2" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="144" ht="18.75" spans="1:3">
-      <c r="A144" s="5">
-        <v>4620000002</v>
-      </c>
-      <c r="B144" s="2" t="s">
+      <c r="C144" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="145" ht="18.75" spans="1:3">
+      <c r="A145" s="2">
+        <v>4471000000</v>
+      </c>
+      <c r="B145" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="C144" s="2" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="145" ht="18.75" spans="1:3">
-      <c r="A145" s="5">
-        <v>4620000003</v>
-      </c>
-      <c r="B145" s="2" t="s">
+      <c r="C145" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="146" ht="18.75" spans="1:3">
+      <c r="A146" s="2">
+        <v>4472000000</v>
+      </c>
+      <c r="B146" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="C145" s="2" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="146" ht="18.75" spans="1:3">
-      <c r="A146" s="5">
-        <v>4620000004</v>
-      </c>
-      <c r="B146" s="2" t="s">
-        <v>149</v>
-      </c>
       <c r="C146" s="2" t="s">
-        <v>146</v>
+        <v>3</v>
       </c>
     </row>
     <row r="147" ht="18.75" spans="1:3">
       <c r="A147" s="5">
-        <v>4620000005</v>
-      </c>
-      <c r="B147" s="3" t="s">
+        <v>4620000001</v>
+      </c>
+      <c r="B147" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="C147" s="2" t="s">
         <v>150</v>
-      </c>
-      <c r="C147" s="2" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="148" ht="18.75" spans="1:3">
       <c r="A148" s="5">
-        <v>4712000000</v>
+        <v>4620000002</v>
       </c>
       <c r="B148" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="C148" s="6" t="s">
-        <v>3</v>
+      <c r="C148" s="2" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="149" ht="18.75" spans="1:3">
       <c r="A149" s="5">
-        <v>4722000000</v>
+        <v>4620000003</v>
       </c>
       <c r="B149" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="C149" s="6" t="s">
-        <v>3</v>
+      <c r="C149" s="2" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="150" ht="18.75" spans="1:3">
-      <c r="A150" s="2">
-        <v>5200000000</v>
+      <c r="A150" s="5">
+        <v>4620000004</v>
       </c>
       <c r="B150" s="2" t="s">
         <v>153</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>16</v>
+        <v>150</v>
       </c>
     </row>
     <row r="151" ht="18.75" spans="1:3">
-      <c r="A151" s="2">
-        <v>5700000000</v>
-      </c>
-      <c r="B151" s="2" t="s">
+      <c r="A151" s="5">
+        <v>4620000005</v>
+      </c>
+      <c r="B151" s="3" t="s">
         <v>154</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>16</v>
+        <v>150</v>
       </c>
     </row>
     <row r="152" ht="18.75" spans="1:3">
-      <c r="A152" s="2">
-        <v>5810000000</v>
+      <c r="A152" s="5">
+        <v>4712000000</v>
       </c>
       <c r="B152" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="C152" s="2"/>
+      <c r="C152" s="6" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="153" ht="18.75" spans="1:3">
-      <c r="A153" s="2">
-        <v>6033000001</v>
+      <c r="A153" s="5">
+        <v>4722000000</v>
       </c>
       <c r="B153" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="C153" s="2" t="s">
-        <v>157</v>
+      <c r="C153" s="6" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="154" ht="18.75" spans="1:3">
       <c r="A154" s="2">
-        <v>6033000002</v>
+        <v>5200000000</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>157</v>
+        <v>16</v>
       </c>
     </row>
     <row r="155" ht="18.75" spans="1:3">
       <c r="A155" s="2">
-        <v>6033000003</v>
+        <v>5700000000</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>157</v>
+        <v>16</v>
       </c>
     </row>
     <row r="156" ht="18.75" spans="1:3">
       <c r="A156" s="2">
-        <v>6033000004</v>
+        <v>5810000000</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>160</v>
-      </c>
-      <c r="C156" s="2" t="s">
-        <v>157</v>
-      </c>
+        <v>159</v>
+      </c>
+      <c r="C156" s="2"/>
     </row>
     <row r="157" ht="18.75" spans="1:3">
       <c r="A157" s="2">
-        <v>6033000005</v>
+        <v>6033000001</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="158" ht="18.75" spans="1:3">
       <c r="A158" s="2">
-        <v>6033000006</v>
+        <v>6033000002</v>
       </c>
       <c r="B158" s="2" t="s">
         <v>162</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="159" ht="18.75" spans="1:3">
       <c r="A159" s="2">
-        <v>6033000007</v>
+        <v>6033000003</v>
       </c>
       <c r="B159" s="2" t="s">
         <v>163</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="160" ht="18.75" spans="1:3">
       <c r="A160" s="2">
-        <v>6033000008</v>
+        <v>6033000004</v>
       </c>
       <c r="B160" s="2" t="s">
         <v>164</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="161" ht="18.75" spans="1:3">
       <c r="A161" s="2">
-        <v>6033000009</v>
+        <v>6033000005</v>
       </c>
       <c r="B161" s="2" t="s">
         <v>165</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="162" ht="18.75" spans="1:3">
       <c r="A162" s="2">
-        <v>6033000010</v>
+        <v>6033000006</v>
       </c>
       <c r="B162" s="2" t="s">
         <v>166</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="163" ht="18.75" spans="1:3">
       <c r="A163" s="2">
-        <v>6033000011</v>
+        <v>6033000007</v>
       </c>
       <c r="B163" s="2" t="s">
         <v>167</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="164" ht="18.75" spans="1:3">
       <c r="A164" s="2">
-        <v>6033000012</v>
+        <v>6033000008</v>
       </c>
       <c r="B164" s="2" t="s">
         <v>168</v>
       </c>
       <c r="C164" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="165" ht="18.75" spans="1:3">
       <c r="A165" s="2">
-        <v>6033000013</v>
+        <v>6033000009</v>
       </c>
       <c r="B165" s="2" t="s">
         <v>169</v>
       </c>
       <c r="C165" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="166" ht="18.75" spans="1:3">
       <c r="A166" s="2">
-        <v>6033000014</v>
+        <v>6033000010</v>
       </c>
       <c r="B166" s="2" t="s">
         <v>170</v>
       </c>
       <c r="C166" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="167" ht="18.75" spans="1:3">
       <c r="A167" s="2">
-        <v>6033000015</v>
+        <v>6033000011</v>
       </c>
       <c r="B167" s="2" t="s">
         <v>171</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="168" ht="18.75" spans="1:3">
       <c r="A168" s="2">
-        <v>6033000016</v>
+        <v>6033000012</v>
       </c>
       <c r="B168" s="2" t="s">
         <v>172</v>
       </c>
       <c r="C168" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="169" ht="18.75" spans="1:3">
       <c r="A169" s="2">
-        <v>6033000017</v>
+        <v>6033000013</v>
       </c>
       <c r="B169" s="2" t="s">
         <v>173</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="170" ht="18.75" spans="1:3">
       <c r="A170" s="2">
-        <v>6033000018</v>
+        <v>6033000014</v>
       </c>
       <c r="B170" s="2" t="s">
         <v>174</v>
       </c>
       <c r="C170" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="171" ht="18.75" spans="1:3">
       <c r="A171" s="2">
-        <v>6033000019</v>
+        <v>6033000015</v>
       </c>
       <c r="B171" s="2" t="s">
         <v>175</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="172" ht="18.75" spans="1:3">
       <c r="A172" s="2">
-        <v>6033000020</v>
+        <v>6033000016</v>
       </c>
       <c r="B172" s="2" t="s">
         <v>176</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="173" ht="18.75" spans="1:3">
       <c r="A173" s="2">
-        <v>6033000021</v>
+        <v>6033000017</v>
       </c>
       <c r="B173" s="2" t="s">
         <v>177</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="174" ht="18.75" spans="1:3">
       <c r="A174" s="2">
-        <v>6033000022</v>
+        <v>6033000018</v>
       </c>
       <c r="B174" s="2" t="s">
         <v>178</v>
       </c>
       <c r="C174" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="175" ht="18.75" spans="1:3">
       <c r="A175" s="2">
-        <v>6033000023</v>
+        <v>6033000019</v>
       </c>
       <c r="B175" s="2" t="s">
         <v>179</v>
       </c>
       <c r="C175" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="176" ht="18.75" spans="1:3">
       <c r="A176" s="2">
-        <v>6033000024</v>
+        <v>6033000020</v>
       </c>
       <c r="B176" s="2" t="s">
         <v>180</v>
       </c>
       <c r="C176" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="177" ht="18.75" spans="1:3">
       <c r="A177" s="2">
-        <v>6033000025</v>
+        <v>6033000021</v>
       </c>
       <c r="B177" s="2" t="s">
         <v>181</v>
       </c>
       <c r="C177" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="178" ht="18.75" spans="1:3">
       <c r="A178" s="2">
-        <v>6033000026</v>
+        <v>6033000022</v>
       </c>
       <c r="B178" s="2" t="s">
         <v>182</v>
       </c>
       <c r="C178" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="179" ht="18.75" spans="1:3">
       <c r="A179" s="2">
-        <v>6033000027</v>
+        <v>6033000023</v>
       </c>
       <c r="B179" s="2" t="s">
         <v>183</v>
       </c>
       <c r="C179" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="180" ht="18.75" spans="1:3">
       <c r="A180" s="2">
-        <v>6033000028</v>
+        <v>6033000024</v>
       </c>
       <c r="B180" s="2" t="s">
         <v>184</v>
       </c>
       <c r="C180" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="181" ht="18.75" spans="1:3">
       <c r="A181" s="2">
-        <v>6033000029</v>
+        <v>6033000025</v>
       </c>
       <c r="B181" s="2" t="s">
         <v>185</v>
       </c>
       <c r="C181" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="182" ht="18.75" spans="1:3">
       <c r="A182" s="2">
-        <v>6033000030</v>
+        <v>6033000026</v>
       </c>
       <c r="B182" s="2" t="s">
         <v>186</v>
       </c>
       <c r="C182" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="183" ht="18.75" spans="1:3">
       <c r="A183" s="2">
-        <v>6033000031</v>
+        <v>6033000027</v>
       </c>
       <c r="B183" s="2" t="s">
         <v>187</v>
       </c>
       <c r="C183" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="184" ht="18.75" spans="1:3">
       <c r="A184" s="2">
-        <v>6033000032</v>
+        <v>6033000028</v>
       </c>
       <c r="B184" s="2" t="s">
         <v>188</v>
       </c>
       <c r="C184" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="185" ht="18.75" spans="1:3">
       <c r="A185" s="2">
-        <v>6033000033</v>
+        <v>6033000029</v>
       </c>
       <c r="B185" s="2" t="s">
         <v>189</v>
       </c>
       <c r="C185" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="186" ht="18.75" spans="1:3">
       <c r="A186" s="2">
-        <v>6033000034</v>
+        <v>6033000030</v>
       </c>
       <c r="B186" s="2" t="s">
         <v>190</v>
       </c>
       <c r="C186" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="187" ht="18.75" spans="1:3">
       <c r="A187" s="2">
-        <v>6033000035</v>
+        <v>6033000031</v>
       </c>
       <c r="B187" s="2" t="s">
         <v>191</v>
       </c>
       <c r="C187" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="188" ht="18.75" spans="1:3">
       <c r="A188" s="2">
-        <v>6033000036</v>
+        <v>6033000032</v>
       </c>
       <c r="B188" s="2" t="s">
         <v>192</v>
       </c>
       <c r="C188" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="189" ht="18.75" spans="1:3">
       <c r="A189" s="2">
-        <v>6033000037</v>
+        <v>6033000033</v>
       </c>
       <c r="B189" s="2" t="s">
         <v>193</v>
       </c>
       <c r="C189" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="190" ht="18.75" spans="1:3">
       <c r="A190" s="2">
-        <v>6033000038</v>
+        <v>6033000034</v>
       </c>
       <c r="B190" s="2" t="s">
         <v>194</v>
       </c>
       <c r="C190" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="191" ht="18.75" spans="1:3">
-      <c r="A191" s="3">
-        <v>6033000039</v>
+      <c r="A191" s="2">
+        <v>6033000035</v>
       </c>
       <c r="B191" s="2" t="s">
         <v>195</v>
       </c>
       <c r="C191" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="192" ht="18.75" spans="1:3">
       <c r="A192" s="2">
-        <v>6033000040</v>
+        <v>6033000036</v>
       </c>
       <c r="B192" s="2" t="s">
         <v>196</v>
       </c>
       <c r="C192" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="193" ht="18.75" spans="1:3">
-      <c r="A193" s="3">
-        <v>6033000041</v>
+      <c r="A193" s="2">
+        <v>6033000037</v>
       </c>
       <c r="B193" s="2" t="s">
         <v>197</v>
       </c>
       <c r="C193" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="194" ht="18.75" spans="1:3">
       <c r="A194" s="2">
-        <v>6047000001</v>
+        <v>6033000038</v>
       </c>
       <c r="B194" s="2" t="s">
         <v>198</v>
       </c>
       <c r="C194" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="195" ht="18.75" spans="1:3">
-      <c r="A195" s="2">
-        <v>6047000002</v>
+      <c r="A195" s="3">
+        <v>6033000039</v>
       </c>
       <c r="B195" s="2" t="s">
         <v>199</v>
       </c>
       <c r="C195" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="196" ht="18.75" spans="1:3">
       <c r="A196" s="2">
-        <v>6047000003</v>
+        <v>6033000040</v>
       </c>
       <c r="B196" s="2" t="s">
         <v>200</v>
       </c>
       <c r="C196" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="197" ht="18.75" spans="1:3">
-      <c r="A197" s="2">
-        <v>6047000004</v>
+      <c r="A197" s="3">
+        <v>6033000041</v>
       </c>
       <c r="B197" s="2" t="s">
         <v>201</v>
       </c>
       <c r="C197" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="198" ht="18.75" spans="1:3">
       <c r="A198" s="2">
-        <v>6047000005</v>
+        <v>6047000001</v>
       </c>
       <c r="B198" s="2" t="s">
         <v>202</v>
       </c>
       <c r="C198" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="199" ht="18.75" spans="1:3">
       <c r="A199" s="2">
-        <v>6047000006</v>
+        <v>6047000002</v>
       </c>
       <c r="B199" s="2" t="s">
         <v>203</v>
       </c>
       <c r="C199" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="200" ht="18.75" spans="1:3">
       <c r="A200" s="2">
-        <v>6047000007</v>
+        <v>6047000003</v>
       </c>
       <c r="B200" s="2" t="s">
         <v>204</v>
       </c>
       <c r="C200" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="201" ht="18.75" spans="1:3">
       <c r="A201" s="2">
-        <v>6047000008</v>
+        <v>6047000004</v>
       </c>
       <c r="B201" s="2" t="s">
         <v>205</v>
       </c>
       <c r="C201" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="202" ht="18.75" spans="1:3">
       <c r="A202" s="2">
-        <v>6047000009</v>
+        <v>6047000005</v>
       </c>
       <c r="B202" s="2" t="s">
         <v>206</v>
       </c>
       <c r="C202" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="203" ht="18.75" spans="1:3">
       <c r="A203" s="2">
-        <v>6047000010</v>
+        <v>6047000006</v>
       </c>
       <c r="B203" s="2" t="s">
         <v>207</v>
       </c>
       <c r="C203" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="204" ht="18.75" spans="1:3">
       <c r="A204" s="2">
-        <v>6047000011</v>
+        <v>6047000007</v>
       </c>
       <c r="B204" s="2" t="s">
         <v>208</v>
       </c>
       <c r="C204" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="205" ht="18.75" spans="1:3">
       <c r="A205" s="2">
-        <v>6047000012</v>
+        <v>6047000008</v>
       </c>
       <c r="B205" s="2" t="s">
         <v>209</v>
       </c>
       <c r="C205" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="206" ht="18.75" spans="1:3">
       <c r="A206" s="2">
-        <v>6055000001</v>
+        <v>6047000009</v>
       </c>
       <c r="B206" s="2" t="s">
         <v>210</v>
       </c>
       <c r="C206" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="207" ht="18.75" spans="1:3">
       <c r="A207" s="2">
-        <v>6055000002</v>
+        <v>6047000010</v>
       </c>
       <c r="B207" s="2" t="s">
         <v>211</v>
       </c>
       <c r="C207" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="208" ht="18.75" spans="1:3">
       <c r="A208" s="2">
-        <v>6055000003</v>
+        <v>6047000011</v>
       </c>
       <c r="B208" s="2" t="s">
         <v>212</v>
       </c>
       <c r="C208" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="209" ht="18.75" spans="1:3">
       <c r="A209" s="2">
-        <v>6055000004</v>
+        <v>6047000012</v>
       </c>
       <c r="B209" s="2" t="s">
         <v>213</v>
       </c>
       <c r="C209" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="210" ht="18.75" spans="1:3">
       <c r="A210" s="2">
-        <v>6055000005</v>
+        <v>6055000001</v>
       </c>
       <c r="B210" s="2" t="s">
         <v>214</v>
       </c>
       <c r="C210" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="211" ht="18.75" spans="1:3">
       <c r="A211" s="2">
-        <v>6055000006</v>
+        <v>6055000002</v>
       </c>
       <c r="B211" s="2" t="s">
         <v>215</v>
       </c>
       <c r="C211" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="212" ht="18.75" spans="1:3">
       <c r="A212" s="2">
-        <v>6055000007</v>
+        <v>6055000003</v>
       </c>
       <c r="B212" s="2" t="s">
         <v>216</v>
       </c>
       <c r="C212" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="213" ht="18.75" spans="1:3">
       <c r="A213" s="2">
-        <v>6055000008</v>
+        <v>6055000004</v>
       </c>
       <c r="B213" s="2" t="s">
         <v>217</v>
       </c>
       <c r="C213" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="214" ht="18.75" spans="1:3">
       <c r="A214" s="2">
-        <v>6055000009</v>
+        <v>6055000005</v>
       </c>
       <c r="B214" s="2" t="s">
         <v>218</v>
       </c>
       <c r="C214" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="215" ht="18.75" spans="1:3">
       <c r="A215" s="2">
-        <v>6055000010</v>
+        <v>6055000006</v>
       </c>
       <c r="B215" s="2" t="s">
         <v>219</v>
       </c>
       <c r="C215" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="216" ht="18.75" spans="1:3">
       <c r="A216" s="2">
-        <v>6055000011</v>
+        <v>6055000007</v>
       </c>
       <c r="B216" s="2" t="s">
         <v>220</v>
       </c>
       <c r="C216" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="217" ht="18.75" spans="1:3">
       <c r="A217" s="2">
-        <v>6055000012</v>
+        <v>6055000008</v>
       </c>
       <c r="B217" s="2" t="s">
         <v>221</v>
       </c>
       <c r="C217" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="218" ht="18.75" spans="1:3">
       <c r="A218" s="2">
-        <v>6055000013</v>
+        <v>6055000009</v>
       </c>
       <c r="B218" s="2" t="s">
         <v>222</v>
       </c>
       <c r="C218" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="219" ht="18.75" spans="1:3">
       <c r="A219" s="2">
-        <v>6056000000</v>
+        <v>6055000010</v>
       </c>
       <c r="B219" s="2" t="s">
         <v>223</v>
       </c>
       <c r="C219" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="220" ht="18.75" spans="1:3">
       <c r="A220" s="2">
-        <v>6056000001</v>
+        <v>6055000011</v>
       </c>
       <c r="B220" s="2" t="s">
         <v>224</v>
       </c>
       <c r="C220" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="221" ht="18.75" spans="1:3">
       <c r="A221" s="2">
-        <v>6056000002</v>
+        <v>6055000012</v>
       </c>
       <c r="B221" s="2" t="s">
         <v>225</v>
       </c>
       <c r="C221" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="222" ht="18.75" spans="1:3">
       <c r="A222" s="2">
-        <v>6056000003</v>
+        <v>6055000013</v>
       </c>
       <c r="B222" s="2" t="s">
         <v>226</v>
       </c>
       <c r="C222" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="223" ht="18.75" spans="1:3">
       <c r="A223" s="2">
-        <v>6056000004</v>
+        <v>6056000000</v>
       </c>
       <c r="B223" s="2" t="s">
         <v>227</v>
       </c>
       <c r="C223" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="224" ht="18.75" spans="1:3">
       <c r="A224" s="2">
-        <v>6056000005</v>
+        <v>6056000001</v>
       </c>
       <c r="B224" s="2" t="s">
         <v>228</v>
       </c>
       <c r="C224" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="225" ht="18.75" spans="1:3">
       <c r="A225" s="2">
-        <v>6056000006</v>
+        <v>6056000002</v>
       </c>
       <c r="B225" s="2" t="s">
         <v>229</v>
       </c>
       <c r="C225" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="226" ht="18.75" spans="1:3">
       <c r="A226" s="2">
-        <v>6056000007</v>
+        <v>6056000003</v>
       </c>
       <c r="B226" s="2" t="s">
         <v>230</v>
       </c>
       <c r="C226" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="227" ht="18.75" spans="1:3">
       <c r="A227" s="2">
-        <v>6056000008</v>
+        <v>6056000004</v>
       </c>
       <c r="B227" s="2" t="s">
         <v>231</v>
       </c>
       <c r="C227" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="228" ht="18.75" spans="1:3">
       <c r="A228" s="2">
-        <v>6056000009</v>
+        <v>6056000005</v>
       </c>
       <c r="B228" s="2" t="s">
         <v>232</v>
       </c>
       <c r="C228" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="229" ht="18.75" spans="1:3">
       <c r="A229" s="2">
-        <v>6056000010</v>
+        <v>6056000006</v>
       </c>
       <c r="B229" s="2" t="s">
         <v>233</v>
       </c>
       <c r="C229" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="230" ht="18.75" spans="1:3">
       <c r="A230" s="2">
-        <v>6056000011</v>
+        <v>6056000007</v>
       </c>
       <c r="B230" s="2" t="s">
         <v>234</v>
       </c>
       <c r="C230" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="231" ht="18.75" spans="1:3">
       <c r="A231" s="2">
-        <v>6056000012</v>
+        <v>6056000008</v>
       </c>
       <c r="B231" s="2" t="s">
         <v>235</v>
       </c>
       <c r="C231" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="232" ht="18.75" spans="1:3">
       <c r="A232" s="2">
-        <v>6056000013</v>
+        <v>6056000009</v>
       </c>
       <c r="B232" s="2" t="s">
         <v>236</v>
       </c>
       <c r="C232" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="233" ht="18.75" spans="1:3">
       <c r="A233" s="2">
-        <v>6056000014</v>
+        <v>6056000010</v>
       </c>
       <c r="B233" s="2" t="s">
         <v>237</v>
       </c>
       <c r="C233" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="234" ht="18.75" spans="1:3">
       <c r="A234" s="2">
-        <v>6056000015</v>
+        <v>6056000011</v>
       </c>
       <c r="B234" s="2" t="s">
         <v>238</v>
       </c>
       <c r="C234" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="235" ht="18.75" spans="1:3">
       <c r="A235" s="2">
-        <v>6056000016</v>
+        <v>6056000012</v>
       </c>
       <c r="B235" s="2" t="s">
         <v>239</v>
       </c>
       <c r="C235" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="236" ht="18.75" spans="1:3">
       <c r="A236" s="2">
-        <v>6056000017</v>
+        <v>6056000013</v>
       </c>
       <c r="B236" s="2" t="s">
         <v>240</v>
       </c>
       <c r="C236" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="237" ht="18.75" spans="1:3">
       <c r="A237" s="2">
-        <v>6056000018</v>
+        <v>6056000014</v>
       </c>
       <c r="B237" s="2" t="s">
         <v>241</v>
       </c>
       <c r="C237" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="238" ht="18.75" spans="1:3">
       <c r="A238" s="2">
-        <v>6056000019</v>
+        <v>6056000015</v>
       </c>
       <c r="B238" s="2" t="s">
         <v>242</v>
       </c>
       <c r="C238" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="239" ht="18.75" spans="1:3">
       <c r="A239" s="2">
-        <v>6056000020</v>
+        <v>6056000016</v>
       </c>
       <c r="B239" s="2" t="s">
         <v>243</v>
       </c>
       <c r="C239" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="240" ht="18.75" spans="1:3">
       <c r="A240" s="2">
-        <v>6056000021</v>
+        <v>6056000017</v>
       </c>
       <c r="B240" s="2" t="s">
         <v>244</v>
       </c>
       <c r="C240" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="241" ht="18.75" spans="1:3">
       <c r="A241" s="2">
-        <v>6056000022</v>
+        <v>6056000018</v>
       </c>
       <c r="B241" s="2" t="s">
         <v>245</v>
       </c>
       <c r="C241" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="242" ht="18.75" spans="1:3">
       <c r="A242" s="2">
-        <v>6056000023</v>
+        <v>6056000019</v>
       </c>
       <c r="B242" s="2" t="s">
         <v>246</v>
       </c>
       <c r="C242" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="243" ht="18.75" spans="1:3">
       <c r="A243" s="2">
-        <v>6056000024</v>
+        <v>6056000020</v>
       </c>
       <c r="B243" s="2" t="s">
         <v>247</v>
       </c>
       <c r="C243" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="244" ht="18.75" spans="1:3">
       <c r="A244" s="2">
-        <v>6056000025</v>
+        <v>6056000021</v>
       </c>
       <c r="B244" s="2" t="s">
         <v>248</v>
       </c>
       <c r="C244" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="245" ht="18.75" spans="1:3">
       <c r="A245" s="2">
-        <v>6056000026</v>
+        <v>6056000022</v>
       </c>
       <c r="B245" s="2" t="s">
         <v>249</v>
       </c>
       <c r="C245" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="246" ht="18.75" spans="1:3">
       <c r="A246" s="2">
-        <v>6056000027</v>
+        <v>6056000023</v>
       </c>
       <c r="B246" s="2" t="s">
         <v>250</v>
       </c>
       <c r="C246" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="247" ht="18.75" spans="1:3">
       <c r="A247" s="2">
-        <v>6056000028</v>
+        <v>6056000024</v>
       </c>
       <c r="B247" s="2" t="s">
         <v>251</v>
       </c>
       <c r="C247" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="248" ht="18.75" spans="1:3">
       <c r="A248" s="2">
-        <v>6056000029</v>
+        <v>6056000025</v>
       </c>
       <c r="B248" s="2" t="s">
         <v>252</v>
       </c>
       <c r="C248" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="249" ht="18.75" spans="1:3">
       <c r="A249" s="2">
-        <v>6056000030</v>
+        <v>6056000026</v>
       </c>
       <c r="B249" s="2" t="s">
         <v>253</v>
       </c>
       <c r="C249" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="250" ht="18.75" spans="1:3">
       <c r="A250" s="2">
-        <v>6056000031</v>
+        <v>6056000027</v>
       </c>
       <c r="B250" s="2" t="s">
         <v>254</v>
       </c>
       <c r="C250" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="251" ht="18.75" spans="1:3">
       <c r="A251" s="2">
-        <v>6056000032</v>
+        <v>6056000028</v>
       </c>
       <c r="B251" s="2" t="s">
         <v>255</v>
       </c>
       <c r="C251" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="252" ht="18.75" spans="1:3">
       <c r="A252" s="2">
-        <v>6056000033</v>
+        <v>6056000029</v>
       </c>
       <c r="B252" s="2" t="s">
         <v>256</v>
       </c>
       <c r="C252" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="253" ht="18.75" spans="1:3">
       <c r="A253" s="2">
-        <v>6056000034</v>
+        <v>6056000030</v>
       </c>
       <c r="B253" s="2" t="s">
         <v>257</v>
       </c>
       <c r="C253" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="254" ht="18.75" spans="1:3">
       <c r="A254" s="2">
-        <v>6056000035</v>
+        <v>6056000031</v>
       </c>
       <c r="B254" s="2" t="s">
         <v>258</v>
       </c>
       <c r="C254" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="255" ht="18.75" spans="1:3">
       <c r="A255" s="2">
-        <v>6056000036</v>
+        <v>6056000032</v>
       </c>
       <c r="B255" s="2" t="s">
         <v>259</v>
       </c>
       <c r="C255" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="256" ht="18.75" spans="1:3">
       <c r="A256" s="2">
-        <v>6056000037</v>
+        <v>6056000033</v>
       </c>
       <c r="B256" s="2" t="s">
         <v>260</v>
       </c>
       <c r="C256" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="257" ht="18.75" spans="1:3">
       <c r="A257" s="2">
-        <v>6056000038</v>
+        <v>6056000034</v>
       </c>
       <c r="B257" s="2" t="s">
         <v>261</v>
       </c>
       <c r="C257" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="258" ht="18.75" spans="1:3">
       <c r="A258" s="2">
-        <v>6056000039</v>
+        <v>6056000035</v>
       </c>
       <c r="B258" s="2" t="s">
         <v>262</v>
       </c>
       <c r="C258" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="259" ht="18.75" spans="1:3">
       <c r="A259" s="2">
-        <v>6056000040</v>
+        <v>6056000036</v>
       </c>
       <c r="B259" s="2" t="s">
-        <v>222</v>
+        <v>263</v>
       </c>
       <c r="C259" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="260" ht="18.75" spans="1:3">
       <c r="A260" s="2">
-        <v>6056000041</v>
+        <v>6056000037</v>
       </c>
       <c r="B260" s="2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C260" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="261" ht="18.75" spans="1:3">
       <c r="A261" s="2">
-        <v>6056000042</v>
+        <v>6056000038</v>
       </c>
       <c r="B261" s="2" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C261" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="262" ht="18.75" spans="1:3">
       <c r="A262" s="2">
-        <v>6056000043</v>
+        <v>6056000039</v>
       </c>
       <c r="B262" s="2" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C262" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="263" ht="18.75" spans="1:3">
       <c r="A263" s="2">
-        <v>6056000044</v>
+        <v>6056000040</v>
       </c>
       <c r="B263" s="2" t="s">
-        <v>266</v>
+        <v>226</v>
       </c>
       <c r="C263" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="264" ht="18.75" spans="1:3">
       <c r="A264" s="2">
-        <v>6056000045</v>
+        <v>6056000041</v>
       </c>
       <c r="B264" s="2" t="s">
         <v>267</v>
       </c>
       <c r="C264" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="265" ht="18.75" spans="1:3">
       <c r="A265" s="2">
-        <v>6056000046</v>
+        <v>6056000042</v>
       </c>
       <c r="B265" s="2" t="s">
         <v>268</v>
       </c>
       <c r="C265" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="266" ht="18.75" spans="1:3">
       <c r="A266" s="2">
-        <v>6056000047</v>
+        <v>6056000043</v>
       </c>
       <c r="B266" s="2" t="s">
         <v>269</v>
       </c>
       <c r="C266" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="267" ht="18.75" spans="1:3">
       <c r="A267" s="2">
-        <v>6056000048</v>
+        <v>6056000044</v>
       </c>
       <c r="B267" s="2" t="s">
         <v>270</v>
       </c>
       <c r="C267" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="268" ht="18.75" spans="1:3">
       <c r="A268" s="2">
-        <v>6056000049</v>
+        <v>6056000045</v>
       </c>
       <c r="B268" s="2" t="s">
         <v>271</v>
       </c>
       <c r="C268" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="269" ht="18.75" spans="1:3">
       <c r="A269" s="2">
-        <v>6056000050</v>
+        <v>6056000046</v>
       </c>
       <c r="B269" s="2" t="s">
         <v>272</v>
       </c>
       <c r="C269" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="270" ht="18.75" spans="1:3">
       <c r="A270" s="2">
-        <v>6056000051</v>
+        <v>6056000047</v>
       </c>
       <c r="B270" s="2" t="s">
         <v>273</v>
       </c>
       <c r="C270" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="271" ht="18.75" spans="1:3">
       <c r="A271" s="2">
-        <v>6056000052</v>
+        <v>6056000048</v>
       </c>
       <c r="B271" s="2" t="s">
         <v>274</v>
       </c>
       <c r="C271" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="272" ht="18.75" spans="1:3">
       <c r="A272" s="2">
-        <v>6056000053</v>
+        <v>6056000049</v>
       </c>
       <c r="B272" s="2" t="s">
         <v>275</v>
       </c>
       <c r="C272" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="273" ht="18.75" spans="1:3">
       <c r="A273" s="2">
-        <v>6056000054</v>
+        <v>6056000050</v>
       </c>
       <c r="B273" s="2" t="s">
         <v>276</v>
       </c>
       <c r="C273" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="274" ht="18.75" spans="1:3">
       <c r="A274" s="2">
-        <v>6056000055</v>
+        <v>6056000051</v>
       </c>
       <c r="B274" s="2" t="s">
         <v>277</v>
       </c>
       <c r="C274" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="275" ht="18.75" spans="1:3">
       <c r="A275" s="2">
-        <v>6056000056</v>
+        <v>6056000052</v>
       </c>
       <c r="B275" s="2" t="s">
         <v>278</v>
       </c>
       <c r="C275" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="276" ht="18.75" spans="1:3">
       <c r="A276" s="2">
-        <v>6056000057</v>
+        <v>6056000053</v>
       </c>
       <c r="B276" s="2" t="s">
         <v>279</v>
       </c>
       <c r="C276" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="277" ht="18.75" spans="1:3">
       <c r="A277" s="2">
-        <v>6056000058</v>
+        <v>6056000054</v>
       </c>
       <c r="B277" s="2" t="s">
         <v>280</v>
       </c>
       <c r="C277" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="278" ht="18.75" spans="1:3">
       <c r="A278" s="2">
-        <v>6056000059</v>
+        <v>6056000055</v>
       </c>
       <c r="B278" s="2" t="s">
         <v>281</v>
       </c>
       <c r="C278" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="279" ht="18.75" spans="1:3">
       <c r="A279" s="2">
-        <v>6080000001</v>
+        <v>6056000056</v>
       </c>
       <c r="B279" s="2" t="s">
         <v>282</v>
       </c>
       <c r="C279" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="280" ht="18.75" spans="1:3">
       <c r="A280" s="2">
-        <v>6080000002</v>
+        <v>6056000057</v>
       </c>
       <c r="B280" s="2" t="s">
         <v>283</v>
       </c>
       <c r="C280" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="281" ht="18.75" spans="1:3">
       <c r="A281" s="2">
-        <v>6080000003</v>
+        <v>6056000058</v>
       </c>
       <c r="B281" s="2" t="s">
         <v>284</v>
       </c>
       <c r="C281" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="282" ht="18.75" spans="1:3">
       <c r="A282" s="2">
-        <v>6080000004</v>
+        <v>6056000059</v>
       </c>
       <c r="B282" s="2" t="s">
         <v>285</v>
       </c>
       <c r="C282" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="283" ht="18.75" spans="1:3">
       <c r="A283" s="2">
-        <v>6080000005</v>
+        <v>6080000001</v>
       </c>
       <c r="B283" s="2" t="s">
         <v>286</v>
       </c>
       <c r="C283" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="284" ht="18.75" spans="1:3">
-      <c r="A284" s="7">
-        <v>6140000000</v>
-      </c>
-      <c r="B284" s="7" t="s">
+      <c r="A284" s="2">
+        <v>6080000002</v>
+      </c>
+      <c r="B284" s="2" t="s">
         <v>287</v>
       </c>
       <c r="C284" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="285" ht="18.75" spans="1:3">
       <c r="A285" s="2">
-        <v>6220000000</v>
+        <v>6080000003</v>
       </c>
       <c r="B285" s="2" t="s">
         <v>288</v>
       </c>
       <c r="C285" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="286" ht="18.75" spans="1:3">
       <c r="A286" s="2">
-        <v>6223000001</v>
+        <v>6080000004</v>
       </c>
       <c r="B286" s="2" t="s">
         <v>289</v>
       </c>
       <c r="C286" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="287" ht="18.75" spans="1:3">
       <c r="A287" s="2">
-        <v>6223000002</v>
+        <v>6080000005</v>
       </c>
       <c r="B287" s="2" t="s">
         <v>290</v>
       </c>
       <c r="C287" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="288" ht="18.75" spans="1:3">
-      <c r="A288" s="2">
-        <v>6223000003</v>
-      </c>
-      <c r="B288" s="2" t="s">
+      <c r="A288" s="7">
+        <v>6140000000</v>
+      </c>
+      <c r="B288" s="7" t="s">
         <v>291</v>
       </c>
       <c r="C288" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="289" ht="18.75" spans="1:3">
       <c r="A289" s="2">
-        <v>6223000004</v>
+        <v>6220000000</v>
       </c>
       <c r="B289" s="2" t="s">
         <v>292</v>
       </c>
       <c r="C289" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="290" ht="18.75" spans="1:3">
       <c r="A290" s="2">
-        <v>6223000005</v>
+        <v>6223000001</v>
       </c>
       <c r="B290" s="2" t="s">
         <v>293</v>
       </c>
       <c r="C290" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="291" ht="18.75" spans="1:3">
       <c r="A291" s="2">
-        <v>6223000006</v>
+        <v>6223000002</v>
       </c>
       <c r="B291" s="2" t="s">
         <v>294</v>
       </c>
       <c r="C291" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="292" ht="18.75" spans="1:3">
       <c r="A292" s="2">
-        <v>6223000007</v>
+        <v>6223000003</v>
       </c>
       <c r="B292" s="2" t="s">
         <v>295</v>
       </c>
       <c r="C292" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="293" ht="18.75" spans="1:3">
       <c r="A293" s="2">
-        <v>6223000008</v>
+        <v>6223000004</v>
       </c>
       <c r="B293" s="2" t="s">
         <v>296</v>
       </c>
       <c r="C293" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="294" ht="18.75" spans="1:3">
       <c r="A294" s="2">
-        <v>6223000009</v>
+        <v>6223000005</v>
       </c>
       <c r="B294" s="2" t="s">
         <v>297</v>
       </c>
       <c r="C294" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="295" ht="18.75" spans="1:3">
       <c r="A295" s="2">
-        <v>6240000000</v>
+        <v>6223000006</v>
       </c>
       <c r="B295" s="2" t="s">
         <v>298</v>
       </c>
       <c r="C295" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="296" ht="18.75" spans="1:3">
       <c r="A296" s="2">
-        <v>6240000001</v>
+        <v>6223000007</v>
       </c>
       <c r="B296" s="2" t="s">
         <v>299</v>
       </c>
       <c r="C296" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="297" ht="18.75" spans="1:3">
       <c r="A297" s="2">
-        <v>6240000002</v>
+        <v>6223000008</v>
       </c>
       <c r="B297" s="2" t="s">
         <v>300</v>
       </c>
       <c r="C297" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="298" ht="18.75" spans="1:3">
       <c r="A298" s="2">
-        <v>6240000003</v>
+        <v>6223000009</v>
       </c>
       <c r="B298" s="2" t="s">
         <v>301</v>
       </c>
       <c r="C298" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="299" ht="18.75" spans="1:3">
       <c r="A299" s="2">
-        <v>6240000004</v>
+        <v>6240000000</v>
       </c>
       <c r="B299" s="2" t="s">
         <v>302</v>
       </c>
       <c r="C299" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="300" ht="18.75" spans="1:3">
       <c r="A300" s="2">
-        <v>6240000005</v>
+        <v>6240000001</v>
       </c>
       <c r="B300" s="2" t="s">
         <v>303</v>
       </c>
       <c r="C300" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="301" ht="18.75" spans="1:3">
       <c r="A301" s="2">
-        <v>6240000006</v>
+        <v>6240000002</v>
       </c>
       <c r="B301" s="2" t="s">
         <v>304</v>
       </c>
       <c r="C301" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="302" ht="18.75" spans="1:3">
       <c r="A302" s="2">
-        <v>6240000007</v>
+        <v>6240000003</v>
       </c>
       <c r="B302" s="2" t="s">
         <v>305</v>
       </c>
       <c r="C302" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="303" ht="18.75" spans="1:3">
       <c r="A303" s="2">
-        <v>6240000008</v>
+        <v>6240000004</v>
       </c>
       <c r="B303" s="2" t="s">
         <v>306</v>
       </c>
       <c r="C303" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="304" ht="18.75" spans="1:3">
       <c r="A304" s="2">
-        <v>6240000009</v>
+        <v>6240000005</v>
       </c>
       <c r="B304" s="2" t="s">
         <v>307</v>
       </c>
       <c r="C304" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="305" ht="18.75" spans="1:3">
       <c r="A305" s="2">
-        <v>6288000000</v>
+        <v>6240000006</v>
       </c>
       <c r="B305" s="2" t="s">
         <v>308</v>
       </c>
       <c r="C305" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="306" ht="18.75" spans="1:3">
       <c r="A306" s="2">
-        <v>6384000001</v>
+        <v>6240000007</v>
       </c>
       <c r="B306" s="2" t="s">
         <v>309</v>
       </c>
       <c r="C306" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="307" ht="18.75" spans="1:3">
       <c r="A307" s="2">
-        <v>6384000002</v>
+        <v>6240000008</v>
       </c>
       <c r="B307" s="2" t="s">
         <v>310</v>
       </c>
       <c r="C307" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="308" ht="18.75" spans="1:3">
       <c r="A308" s="2">
-        <v>6500000000</v>
+        <v>6240000009</v>
       </c>
       <c r="B308" s="2" t="s">
         <v>311</v>
       </c>
       <c r="C308" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="309" ht="18.75" spans="1:3">
       <c r="A309" s="2">
-        <v>6620000000</v>
+        <v>6288000000</v>
       </c>
       <c r="B309" s="2" t="s">
         <v>312</v>
       </c>
       <c r="C309" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="310" ht="18.75" spans="1:3">
       <c r="A310" s="2">
-        <v>6621000001</v>
+        <v>6384000001</v>
       </c>
       <c r="B310" s="2" t="s">
         <v>313</v>
       </c>
       <c r="C310" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="311" ht="18.75" spans="1:3">
       <c r="A311" s="2">
-        <v>6621000002</v>
+        <v>6384000002</v>
       </c>
       <c r="B311" s="2" t="s">
         <v>314</v>
       </c>
       <c r="C311" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="312" ht="18.75" spans="1:3">
       <c r="A312" s="2">
-        <v>6631000000</v>
+        <v>6500000000</v>
       </c>
       <c r="B312" s="2" t="s">
         <v>315</v>
       </c>
       <c r="C312" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="313" ht="18.75" spans="1:3">
       <c r="A313" s="2">
-        <v>6662000000</v>
+        <v>6620000000</v>
       </c>
       <c r="B313" s="2" t="s">
         <v>316</v>
       </c>
       <c r="C313" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="314" ht="18.75" spans="1:3">
       <c r="A314" s="2">
-        <v>6672000000</v>
+        <v>6621000001</v>
       </c>
       <c r="B314" s="2" t="s">
         <v>317</v>
       </c>
       <c r="C314" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="315" ht="18.75" spans="1:3">
       <c r="A315" s="2">
-        <v>6672000001</v>
+        <v>6621000002</v>
       </c>
       <c r="B315" s="2" t="s">
         <v>318</v>
       </c>
       <c r="C315" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="316" ht="18.75" spans="1:3">
       <c r="A316" s="2">
-        <v>6672000002</v>
+        <v>6631000000</v>
       </c>
       <c r="B316" s="2" t="s">
         <v>319</v>
       </c>
       <c r="C316" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="317" ht="18.75" spans="1:3">
       <c r="A317" s="2">
-        <v>6672000003</v>
+        <v>6662000000</v>
       </c>
       <c r="B317" s="2" t="s">
         <v>320</v>
       </c>
       <c r="C317" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="318" ht="18.75" spans="1:3">
       <c r="A318" s="2">
-        <v>6730000000</v>
+        <v>6672000000</v>
       </c>
       <c r="B318" s="2" t="s">
         <v>321</v>
       </c>
       <c r="C318" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="319" ht="18.75" spans="1:3">
       <c r="A319" s="2">
-        <v>6760000000</v>
+        <v>6672000001</v>
       </c>
       <c r="B319" s="2" t="s">
         <v>322</v>
       </c>
       <c r="C319" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="320" ht="18.75" spans="1:3">
       <c r="A320" s="2">
-        <v>6810000000</v>
+        <v>6672000002</v>
       </c>
       <c r="B320" s="2" t="s">
         <v>323</v>
       </c>
       <c r="C320" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="321" ht="18.75" spans="1:3">
       <c r="A321" s="2">
-        <v>7010000001</v>
+        <v>6672000003</v>
       </c>
       <c r="B321" s="2" t="s">
         <v>324</v>
       </c>
       <c r="C321" s="2" t="s">
-        <v>325</v>
+        <v>161</v>
       </c>
     </row>
     <row r="322" ht="18.75" spans="1:3">
       <c r="A322" s="2">
-        <v>7010000002</v>
+        <v>6730000000</v>
       </c>
       <c r="B322" s="2" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C322" s="2" t="s">
-        <v>325</v>
+        <v>161</v>
       </c>
     </row>
     <row r="323" ht="18.75" spans="1:3">
       <c r="A323" s="2">
-        <v>7010000003</v>
+        <v>6760000000</v>
       </c>
       <c r="B323" s="2" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C323" s="2" t="s">
-        <v>325</v>
+        <v>161</v>
       </c>
     </row>
     <row r="324" ht="18.75" spans="1:3">
       <c r="A324" s="2">
-        <v>7010000004</v>
+        <v>6810000000</v>
       </c>
       <c r="B324" s="2" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C324" s="2" t="s">
-        <v>325</v>
+        <v>161</v>
       </c>
     </row>
     <row r="325" ht="18.75" spans="1:3">
       <c r="A325" s="2">
-        <v>7010000005</v>
+        <v>7010000001</v>
       </c>
       <c r="B325" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="C325" s="2" t="s">
         <v>329</v>
-      </c>
-      <c r="C325" s="2" t="s">
-        <v>325</v>
       </c>
     </row>
     <row r="326" ht="18.75" spans="1:3">
       <c r="A326" s="2">
-        <v>7010000006</v>
+        <v>7010000002</v>
       </c>
       <c r="B326" s="2" t="s">
         <v>330</v>
       </c>
       <c r="C326" s="2" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
     <row r="327" ht="18.75" spans="1:3">
       <c r="A327" s="2">
-        <v>7010000007</v>
+        <v>7010000003</v>
       </c>
       <c r="B327" s="2" t="s">
         <v>331</v>
       </c>
       <c r="C327" s="2" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
     <row r="328" ht="18.75" spans="1:3">
       <c r="A328" s="2">
-        <v>7010000008</v>
+        <v>7010000004</v>
       </c>
       <c r="B328" s="2" t="s">
         <v>332</v>
       </c>
       <c r="C328" s="2" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
     <row r="329" ht="18.75" spans="1:3">
       <c r="A329" s="2">
-        <v>7010000009</v>
+        <v>7010000005</v>
       </c>
       <c r="B329" s="2" t="s">
         <v>333</v>
       </c>
       <c r="C329" s="2" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
     <row r="330" ht="18.75" spans="1:3">
       <c r="A330" s="2">
-        <v>7010000010</v>
+        <v>7010000006</v>
       </c>
       <c r="B330" s="2" t="s">
         <v>334</v>
       </c>
       <c r="C330" s="2" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
     <row r="331" ht="18.75" spans="1:3">
       <c r="A331" s="2">
-        <v>7010000011</v>
+        <v>7010000007</v>
       </c>
       <c r="B331" s="2" t="s">
         <v>335</v>
       </c>
       <c r="C331" s="2" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
     <row r="332" ht="18.75" spans="1:3">
       <c r="A332" s="2">
-        <v>7010000012</v>
+        <v>7010000008</v>
       </c>
       <c r="B332" s="2" t="s">
         <v>336</v>
       </c>
       <c r="C332" s="2" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
     <row r="333" ht="18.75" spans="1:3">
       <c r="A333" s="2">
-        <v>7060000000</v>
+        <v>7010000009</v>
       </c>
       <c r="B333" s="2" t="s">
         <v>337</v>
       </c>
       <c r="C333" s="2" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
     <row r="334" ht="18.75" spans="1:3">
       <c r="A334" s="2">
-        <v>7588000000</v>
+        <v>7010000010</v>
       </c>
       <c r="B334" s="2" t="s">
         <v>338</v>
       </c>
       <c r="C334" s="2" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
     <row r="335" ht="18.75" spans="1:3">
       <c r="A335" s="2">
-        <v>7760000000</v>
+        <v>7010000011</v>
       </c>
       <c r="B335" s="2" t="s">
         <v>339</v>
       </c>
       <c r="C335" s="2" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
     <row r="336" ht="18.75" spans="1:3">
       <c r="A336" s="2">
-        <v>7870000000</v>
+        <v>7010000012</v>
       </c>
       <c r="B336" s="2" t="s">
         <v>340</v>
       </c>
       <c r="C336" s="2" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
     <row r="337" ht="18.75" spans="1:3">
-      <c r="A337" s="8">
+      <c r="A337" s="2">
+        <v>7060000000</v>
+      </c>
+      <c r="B337" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="C337" s="2" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="338" ht="18.75" spans="1:3">
+      <c r="A338" s="2">
+        <v>7588000000</v>
+      </c>
+      <c r="B338" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="C338" s="2" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="339" ht="18.75" spans="1:3">
+      <c r="A339" s="2">
+        <v>7760000000</v>
+      </c>
+      <c r="B339" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="C339" s="2" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="340" ht="18.75" spans="1:3">
+      <c r="A340" s="2">
+        <v>7870000000</v>
+      </c>
+      <c r="B340" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="C340" s="2" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="341" ht="18.75" spans="1:3">
+      <c r="A341" s="8">
         <v>8910000000</v>
       </c>
-      <c r="B337" s="8" t="s">
-        <v>341</v>
-      </c>
-      <c r="C337" s="8" t="s">
-        <v>157</v>
+      <c r="B341" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="C341" s="8" t="s">
+        <v>161</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ajout co;pte au plan
</commit_message>
<xml_diff>
--- a/public/PLAN.xlsx
+++ b/public/PLAN.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="675" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="676" uniqueCount="347">
   <si>
     <t>Comptes</t>
   </si>
@@ -507,6 +507,9 @@
   </si>
   <si>
     <t>Acompte Congo Build</t>
+  </si>
+  <si>
+    <t>Acompte ICC / Sous traitant</t>
   </si>
   <si>
     <t>Variation stock salopettes</t>
@@ -2120,7 +2123,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C341"/>
+  <dimension ref="A1:C342"/>
   <sheetFormatPr defaultColWidth="11.4571428571429" defaultRowHeight="15" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="19.4571428571429" customWidth="1"/>
@@ -3830,2037 +3833,2046 @@
     </row>
     <row r="157" ht="18.75" spans="1:3">
       <c r="A157" s="2">
-        <v>6033000001</v>
+        <v>5810000001</v>
       </c>
       <c r="B157" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="C157" s="2" t="s">
-        <v>161</v>
-      </c>
+      <c r="C157" s="2"/>
     </row>
     <row r="158" ht="18.75" spans="1:3">
       <c r="A158" s="2">
-        <v>6033000002</v>
+        <v>6033000001</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="159" ht="18.75" spans="1:3">
       <c r="A159" s="2">
-        <v>6033000003</v>
+        <v>6033000002</v>
       </c>
       <c r="B159" s="2" t="s">
         <v>163</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="160" ht="18.75" spans="1:3">
       <c r="A160" s="2">
-        <v>6033000004</v>
+        <v>6033000003</v>
       </c>
       <c r="B160" s="2" t="s">
         <v>164</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="161" ht="18.75" spans="1:3">
       <c r="A161" s="2">
-        <v>6033000005</v>
+        <v>6033000004</v>
       </c>
       <c r="B161" s="2" t="s">
         <v>165</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="162" ht="18.75" spans="1:3">
       <c r="A162" s="2">
-        <v>6033000006</v>
+        <v>6033000005</v>
       </c>
       <c r="B162" s="2" t="s">
         <v>166</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="163" ht="18.75" spans="1:3">
       <c r="A163" s="2">
-        <v>6033000007</v>
+        <v>6033000006</v>
       </c>
       <c r="B163" s="2" t="s">
         <v>167</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="164" ht="18.75" spans="1:3">
       <c r="A164" s="2">
-        <v>6033000008</v>
+        <v>6033000007</v>
       </c>
       <c r="B164" s="2" t="s">
         <v>168</v>
       </c>
       <c r="C164" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="165" ht="18.75" spans="1:3">
       <c r="A165" s="2">
-        <v>6033000009</v>
+        <v>6033000008</v>
       </c>
       <c r="B165" s="2" t="s">
         <v>169</v>
       </c>
       <c r="C165" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="166" ht="18.75" spans="1:3">
       <c r="A166" s="2">
-        <v>6033000010</v>
+        <v>6033000009</v>
       </c>
       <c r="B166" s="2" t="s">
         <v>170</v>
       </c>
       <c r="C166" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="167" ht="18.75" spans="1:3">
       <c r="A167" s="2">
-        <v>6033000011</v>
+        <v>6033000010</v>
       </c>
       <c r="B167" s="2" t="s">
         <v>171</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="168" ht="18.75" spans="1:3">
       <c r="A168" s="2">
-        <v>6033000012</v>
+        <v>6033000011</v>
       </c>
       <c r="B168" s="2" t="s">
         <v>172</v>
       </c>
       <c r="C168" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="169" ht="18.75" spans="1:3">
       <c r="A169" s="2">
-        <v>6033000013</v>
+        <v>6033000012</v>
       </c>
       <c r="B169" s="2" t="s">
         <v>173</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="170" ht="18.75" spans="1:3">
       <c r="A170" s="2">
-        <v>6033000014</v>
+        <v>6033000013</v>
       </c>
       <c r="B170" s="2" t="s">
         <v>174</v>
       </c>
       <c r="C170" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="171" ht="18.75" spans="1:3">
       <c r="A171" s="2">
-        <v>6033000015</v>
+        <v>6033000014</v>
       </c>
       <c r="B171" s="2" t="s">
         <v>175</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="172" ht="18.75" spans="1:3">
       <c r="A172" s="2">
-        <v>6033000016</v>
+        <v>6033000015</v>
       </c>
       <c r="B172" s="2" t="s">
         <v>176</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="173" ht="18.75" spans="1:3">
       <c r="A173" s="2">
-        <v>6033000017</v>
+        <v>6033000016</v>
       </c>
       <c r="B173" s="2" t="s">
         <v>177</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="174" ht="18.75" spans="1:3">
       <c r="A174" s="2">
-        <v>6033000018</v>
+        <v>6033000017</v>
       </c>
       <c r="B174" s="2" t="s">
         <v>178</v>
       </c>
       <c r="C174" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="175" ht="18.75" spans="1:3">
       <c r="A175" s="2">
-        <v>6033000019</v>
+        <v>6033000018</v>
       </c>
       <c r="B175" s="2" t="s">
         <v>179</v>
       </c>
       <c r="C175" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="176" ht="18.75" spans="1:3">
       <c r="A176" s="2">
-        <v>6033000020</v>
+        <v>6033000019</v>
       </c>
       <c r="B176" s="2" t="s">
         <v>180</v>
       </c>
       <c r="C176" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="177" ht="18.75" spans="1:3">
       <c r="A177" s="2">
-        <v>6033000021</v>
+        <v>6033000020</v>
       </c>
       <c r="B177" s="2" t="s">
         <v>181</v>
       </c>
       <c r="C177" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="178" ht="18.75" spans="1:3">
       <c r="A178" s="2">
-        <v>6033000022</v>
+        <v>6033000021</v>
       </c>
       <c r="B178" s="2" t="s">
         <v>182</v>
       </c>
       <c r="C178" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="179" ht="18.75" spans="1:3">
       <c r="A179" s="2">
-        <v>6033000023</v>
+        <v>6033000022</v>
       </c>
       <c r="B179" s="2" t="s">
         <v>183</v>
       </c>
       <c r="C179" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="180" ht="18.75" spans="1:3">
       <c r="A180" s="2">
-        <v>6033000024</v>
+        <v>6033000023</v>
       </c>
       <c r="B180" s="2" t="s">
         <v>184</v>
       </c>
       <c r="C180" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="181" ht="18.75" spans="1:3">
       <c r="A181" s="2">
-        <v>6033000025</v>
+        <v>6033000024</v>
       </c>
       <c r="B181" s="2" t="s">
         <v>185</v>
       </c>
       <c r="C181" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="182" ht="18.75" spans="1:3">
       <c r="A182" s="2">
-        <v>6033000026</v>
+        <v>6033000025</v>
       </c>
       <c r="B182" s="2" t="s">
         <v>186</v>
       </c>
       <c r="C182" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="183" ht="18.75" spans="1:3">
       <c r="A183" s="2">
-        <v>6033000027</v>
+        <v>6033000026</v>
       </c>
       <c r="B183" s="2" t="s">
         <v>187</v>
       </c>
       <c r="C183" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="184" ht="18.75" spans="1:3">
       <c r="A184" s="2">
-        <v>6033000028</v>
+        <v>6033000027</v>
       </c>
       <c r="B184" s="2" t="s">
         <v>188</v>
       </c>
       <c r="C184" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="185" ht="18.75" spans="1:3">
       <c r="A185" s="2">
-        <v>6033000029</v>
+        <v>6033000028</v>
       </c>
       <c r="B185" s="2" t="s">
         <v>189</v>
       </c>
       <c r="C185" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="186" ht="18.75" spans="1:3">
       <c r="A186" s="2">
-        <v>6033000030</v>
+        <v>6033000029</v>
       </c>
       <c r="B186" s="2" t="s">
         <v>190</v>
       </c>
       <c r="C186" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="187" ht="18.75" spans="1:3">
       <c r="A187" s="2">
-        <v>6033000031</v>
+        <v>6033000030</v>
       </c>
       <c r="B187" s="2" t="s">
         <v>191</v>
       </c>
       <c r="C187" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="188" ht="18.75" spans="1:3">
       <c r="A188" s="2">
-        <v>6033000032</v>
+        <v>6033000031</v>
       </c>
       <c r="B188" s="2" t="s">
         <v>192</v>
       </c>
       <c r="C188" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="189" ht="18.75" spans="1:3">
       <c r="A189" s="2">
-        <v>6033000033</v>
+        <v>6033000032</v>
       </c>
       <c r="B189" s="2" t="s">
         <v>193</v>
       </c>
       <c r="C189" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="190" ht="18.75" spans="1:3">
       <c r="A190" s="2">
-        <v>6033000034</v>
+        <v>6033000033</v>
       </c>
       <c r="B190" s="2" t="s">
         <v>194</v>
       </c>
       <c r="C190" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="191" ht="18.75" spans="1:3">
       <c r="A191" s="2">
-        <v>6033000035</v>
+        <v>6033000034</v>
       </c>
       <c r="B191" s="2" t="s">
         <v>195</v>
       </c>
       <c r="C191" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="192" ht="18.75" spans="1:3">
       <c r="A192" s="2">
-        <v>6033000036</v>
+        <v>6033000035</v>
       </c>
       <c r="B192" s="2" t="s">
         <v>196</v>
       </c>
       <c r="C192" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="193" ht="18.75" spans="1:3">
       <c r="A193" s="2">
-        <v>6033000037</v>
+        <v>6033000036</v>
       </c>
       <c r="B193" s="2" t="s">
         <v>197</v>
       </c>
       <c r="C193" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="194" ht="18.75" spans="1:3">
       <c r="A194" s="2">
-        <v>6033000038</v>
+        <v>6033000037</v>
       </c>
       <c r="B194" s="2" t="s">
         <v>198</v>
       </c>
       <c r="C194" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="195" ht="18.75" spans="1:3">
-      <c r="A195" s="3">
-        <v>6033000039</v>
+      <c r="A195" s="2">
+        <v>6033000038</v>
       </c>
       <c r="B195" s="2" t="s">
         <v>199</v>
       </c>
       <c r="C195" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="196" ht="18.75" spans="1:3">
-      <c r="A196" s="2">
-        <v>6033000040</v>
+      <c r="A196" s="3">
+        <v>6033000039</v>
       </c>
       <c r="B196" s="2" t="s">
         <v>200</v>
       </c>
       <c r="C196" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="197" ht="18.75" spans="1:3">
-      <c r="A197" s="3">
-        <v>6033000041</v>
+      <c r="A197" s="2">
+        <v>6033000040</v>
       </c>
       <c r="B197" s="2" t="s">
         <v>201</v>
       </c>
       <c r="C197" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="198" ht="18.75" spans="1:3">
-      <c r="A198" s="2">
-        <v>6047000001</v>
+      <c r="A198" s="3">
+        <v>6033000041</v>
       </c>
       <c r="B198" s="2" t="s">
         <v>202</v>
       </c>
       <c r="C198" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="199" ht="18.75" spans="1:3">
       <c r="A199" s="2">
-        <v>6047000002</v>
+        <v>6047000001</v>
       </c>
       <c r="B199" s="2" t="s">
         <v>203</v>
       </c>
       <c r="C199" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="200" ht="18.75" spans="1:3">
       <c r="A200" s="2">
-        <v>6047000003</v>
+        <v>6047000002</v>
       </c>
       <c r="B200" s="2" t="s">
         <v>204</v>
       </c>
       <c r="C200" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="201" ht="18.75" spans="1:3">
       <c r="A201" s="2">
-        <v>6047000004</v>
+        <v>6047000003</v>
       </c>
       <c r="B201" s="2" t="s">
         <v>205</v>
       </c>
       <c r="C201" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="202" ht="18.75" spans="1:3">
       <c r="A202" s="2">
-        <v>6047000005</v>
+        <v>6047000004</v>
       </c>
       <c r="B202" s="2" t="s">
         <v>206</v>
       </c>
       <c r="C202" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="203" ht="18.75" spans="1:3">
       <c r="A203" s="2">
-        <v>6047000006</v>
+        <v>6047000005</v>
       </c>
       <c r="B203" s="2" t="s">
         <v>207</v>
       </c>
       <c r="C203" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="204" ht="18.75" spans="1:3">
       <c r="A204" s="2">
-        <v>6047000007</v>
+        <v>6047000006</v>
       </c>
       <c r="B204" s="2" t="s">
         <v>208</v>
       </c>
       <c r="C204" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="205" ht="18.75" spans="1:3">
       <c r="A205" s="2">
-        <v>6047000008</v>
+        <v>6047000007</v>
       </c>
       <c r="B205" s="2" t="s">
         <v>209</v>
       </c>
       <c r="C205" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="206" ht="18.75" spans="1:3">
       <c r="A206" s="2">
-        <v>6047000009</v>
+        <v>6047000008</v>
       </c>
       <c r="B206" s="2" t="s">
         <v>210</v>
       </c>
       <c r="C206" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="207" ht="18.75" spans="1:3">
       <c r="A207" s="2">
-        <v>6047000010</v>
+        <v>6047000009</v>
       </c>
       <c r="B207" s="2" t="s">
         <v>211</v>
       </c>
       <c r="C207" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="208" ht="18.75" spans="1:3">
       <c r="A208" s="2">
-        <v>6047000011</v>
+        <v>6047000010</v>
       </c>
       <c r="B208" s="2" t="s">
         <v>212</v>
       </c>
       <c r="C208" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="209" ht="18.75" spans="1:3">
       <c r="A209" s="2">
-        <v>6047000012</v>
+        <v>6047000011</v>
       </c>
       <c r="B209" s="2" t="s">
         <v>213</v>
       </c>
       <c r="C209" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="210" ht="18.75" spans="1:3">
       <c r="A210" s="2">
-        <v>6055000001</v>
+        <v>6047000012</v>
       </c>
       <c r="B210" s="2" t="s">
         <v>214</v>
       </c>
       <c r="C210" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="211" ht="18.75" spans="1:3">
       <c r="A211" s="2">
-        <v>6055000002</v>
+        <v>6055000001</v>
       </c>
       <c r="B211" s="2" t="s">
         <v>215</v>
       </c>
       <c r="C211" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="212" ht="18.75" spans="1:3">
       <c r="A212" s="2">
-        <v>6055000003</v>
+        <v>6055000002</v>
       </c>
       <c r="B212" s="2" t="s">
         <v>216</v>
       </c>
       <c r="C212" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="213" ht="18.75" spans="1:3">
       <c r="A213" s="2">
-        <v>6055000004</v>
+        <v>6055000003</v>
       </c>
       <c r="B213" s="2" t="s">
         <v>217</v>
       </c>
       <c r="C213" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="214" ht="18.75" spans="1:3">
       <c r="A214" s="2">
-        <v>6055000005</v>
+        <v>6055000004</v>
       </c>
       <c r="B214" s="2" t="s">
         <v>218</v>
       </c>
       <c r="C214" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="215" ht="18.75" spans="1:3">
       <c r="A215" s="2">
-        <v>6055000006</v>
+        <v>6055000005</v>
       </c>
       <c r="B215" s="2" t="s">
         <v>219</v>
       </c>
       <c r="C215" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="216" ht="18.75" spans="1:3">
       <c r="A216" s="2">
-        <v>6055000007</v>
+        <v>6055000006</v>
       </c>
       <c r="B216" s="2" t="s">
         <v>220</v>
       </c>
       <c r="C216" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="217" ht="18.75" spans="1:3">
       <c r="A217" s="2">
-        <v>6055000008</v>
+        <v>6055000007</v>
       </c>
       <c r="B217" s="2" t="s">
         <v>221</v>
       </c>
       <c r="C217" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="218" ht="18.75" spans="1:3">
       <c r="A218" s="2">
-        <v>6055000009</v>
+        <v>6055000008</v>
       </c>
       <c r="B218" s="2" t="s">
         <v>222</v>
       </c>
       <c r="C218" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="219" ht="18.75" spans="1:3">
       <c r="A219" s="2">
-        <v>6055000010</v>
+        <v>6055000009</v>
       </c>
       <c r="B219" s="2" t="s">
         <v>223</v>
       </c>
       <c r="C219" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="220" ht="18.75" spans="1:3">
       <c r="A220" s="2">
-        <v>6055000011</v>
+        <v>6055000010</v>
       </c>
       <c r="B220" s="2" t="s">
         <v>224</v>
       </c>
       <c r="C220" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="221" ht="18.75" spans="1:3">
       <c r="A221" s="2">
-        <v>6055000012</v>
+        <v>6055000011</v>
       </c>
       <c r="B221" s="2" t="s">
         <v>225</v>
       </c>
       <c r="C221" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="222" ht="18.75" spans="1:3">
       <c r="A222" s="2">
-        <v>6055000013</v>
+        <v>6055000012</v>
       </c>
       <c r="B222" s="2" t="s">
         <v>226</v>
       </c>
       <c r="C222" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="223" ht="18.75" spans="1:3">
       <c r="A223" s="2">
-        <v>6056000000</v>
+        <v>6055000013</v>
       </c>
       <c r="B223" s="2" t="s">
         <v>227</v>
       </c>
       <c r="C223" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="224" ht="18.75" spans="1:3">
       <c r="A224" s="2">
-        <v>6056000001</v>
+        <v>6056000000</v>
       </c>
       <c r="B224" s="2" t="s">
         <v>228</v>
       </c>
       <c r="C224" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="225" ht="18.75" spans="1:3">
       <c r="A225" s="2">
-        <v>6056000002</v>
+        <v>6056000001</v>
       </c>
       <c r="B225" s="2" t="s">
         <v>229</v>
       </c>
       <c r="C225" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="226" ht="18.75" spans="1:3">
       <c r="A226" s="2">
-        <v>6056000003</v>
+        <v>6056000002</v>
       </c>
       <c r="B226" s="2" t="s">
         <v>230</v>
       </c>
       <c r="C226" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="227" ht="18.75" spans="1:3">
       <c r="A227" s="2">
-        <v>6056000004</v>
+        <v>6056000003</v>
       </c>
       <c r="B227" s="2" t="s">
         <v>231</v>
       </c>
       <c r="C227" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="228" ht="18.75" spans="1:3">
       <c r="A228" s="2">
-        <v>6056000005</v>
+        <v>6056000004</v>
       </c>
       <c r="B228" s="2" t="s">
         <v>232</v>
       </c>
       <c r="C228" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="229" ht="18.75" spans="1:3">
       <c r="A229" s="2">
-        <v>6056000006</v>
+        <v>6056000005</v>
       </c>
       <c r="B229" s="2" t="s">
         <v>233</v>
       </c>
       <c r="C229" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="230" ht="18.75" spans="1:3">
       <c r="A230" s="2">
-        <v>6056000007</v>
+        <v>6056000006</v>
       </c>
       <c r="B230" s="2" t="s">
         <v>234</v>
       </c>
       <c r="C230" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="231" ht="18.75" spans="1:3">
       <c r="A231" s="2">
-        <v>6056000008</v>
+        <v>6056000007</v>
       </c>
       <c r="B231" s="2" t="s">
         <v>235</v>
       </c>
       <c r="C231" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="232" ht="18.75" spans="1:3">
       <c r="A232" s="2">
-        <v>6056000009</v>
+        <v>6056000008</v>
       </c>
       <c r="B232" s="2" t="s">
         <v>236</v>
       </c>
       <c r="C232" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="233" ht="18.75" spans="1:3">
       <c r="A233" s="2">
-        <v>6056000010</v>
+        <v>6056000009</v>
       </c>
       <c r="B233" s="2" t="s">
         <v>237</v>
       </c>
       <c r="C233" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="234" ht="18.75" spans="1:3">
       <c r="A234" s="2">
-        <v>6056000011</v>
+        <v>6056000010</v>
       </c>
       <c r="B234" s="2" t="s">
         <v>238</v>
       </c>
       <c r="C234" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="235" ht="18.75" spans="1:3">
       <c r="A235" s="2">
-        <v>6056000012</v>
+        <v>6056000011</v>
       </c>
       <c r="B235" s="2" t="s">
         <v>239</v>
       </c>
       <c r="C235" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="236" ht="18.75" spans="1:3">
       <c r="A236" s="2">
-        <v>6056000013</v>
+        <v>6056000012</v>
       </c>
       <c r="B236" s="2" t="s">
         <v>240</v>
       </c>
       <c r="C236" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="237" ht="18.75" spans="1:3">
       <c r="A237" s="2">
-        <v>6056000014</v>
+        <v>6056000013</v>
       </c>
       <c r="B237" s="2" t="s">
         <v>241</v>
       </c>
       <c r="C237" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="238" ht="18.75" spans="1:3">
       <c r="A238" s="2">
-        <v>6056000015</v>
+        <v>6056000014</v>
       </c>
       <c r="B238" s="2" t="s">
         <v>242</v>
       </c>
       <c r="C238" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="239" ht="18.75" spans="1:3">
       <c r="A239" s="2">
-        <v>6056000016</v>
+        <v>6056000015</v>
       </c>
       <c r="B239" s="2" t="s">
         <v>243</v>
       </c>
       <c r="C239" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="240" ht="18.75" spans="1:3">
       <c r="A240" s="2">
-        <v>6056000017</v>
+        <v>6056000016</v>
       </c>
       <c r="B240" s="2" t="s">
         <v>244</v>
       </c>
       <c r="C240" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="241" ht="18.75" spans="1:3">
       <c r="A241" s="2">
-        <v>6056000018</v>
+        <v>6056000017</v>
       </c>
       <c r="B241" s="2" t="s">
         <v>245</v>
       </c>
       <c r="C241" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="242" ht="18.75" spans="1:3">
       <c r="A242" s="2">
-        <v>6056000019</v>
+        <v>6056000018</v>
       </c>
       <c r="B242" s="2" t="s">
         <v>246</v>
       </c>
       <c r="C242" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="243" ht="18.75" spans="1:3">
       <c r="A243" s="2">
-        <v>6056000020</v>
+        <v>6056000019</v>
       </c>
       <c r="B243" s="2" t="s">
         <v>247</v>
       </c>
       <c r="C243" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="244" ht="18.75" spans="1:3">
       <c r="A244" s="2">
-        <v>6056000021</v>
+        <v>6056000020</v>
       </c>
       <c r="B244" s="2" t="s">
         <v>248</v>
       </c>
       <c r="C244" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="245" ht="18.75" spans="1:3">
       <c r="A245" s="2">
-        <v>6056000022</v>
+        <v>6056000021</v>
       </c>
       <c r="B245" s="2" t="s">
         <v>249</v>
       </c>
       <c r="C245" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="246" ht="18.75" spans="1:3">
       <c r="A246" s="2">
-        <v>6056000023</v>
+        <v>6056000022</v>
       </c>
       <c r="B246" s="2" t="s">
         <v>250</v>
       </c>
       <c r="C246" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="247" ht="18.75" spans="1:3">
       <c r="A247" s="2">
-        <v>6056000024</v>
+        <v>6056000023</v>
       </c>
       <c r="B247" s="2" t="s">
         <v>251</v>
       </c>
       <c r="C247" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="248" ht="18.75" spans="1:3">
       <c r="A248" s="2">
-        <v>6056000025</v>
+        <v>6056000024</v>
       </c>
       <c r="B248" s="2" t="s">
         <v>252</v>
       </c>
       <c r="C248" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="249" ht="18.75" spans="1:3">
       <c r="A249" s="2">
-        <v>6056000026</v>
+        <v>6056000025</v>
       </c>
       <c r="B249" s="2" t="s">
         <v>253</v>
       </c>
       <c r="C249" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="250" ht="18.75" spans="1:3">
       <c r="A250" s="2">
-        <v>6056000027</v>
+        <v>6056000026</v>
       </c>
       <c r="B250" s="2" t="s">
         <v>254</v>
       </c>
       <c r="C250" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="251" ht="18.75" spans="1:3">
       <c r="A251" s="2">
-        <v>6056000028</v>
+        <v>6056000027</v>
       </c>
       <c r="B251" s="2" t="s">
         <v>255</v>
       </c>
       <c r="C251" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="252" ht="18.75" spans="1:3">
       <c r="A252" s="2">
-        <v>6056000029</v>
+        <v>6056000028</v>
       </c>
       <c r="B252" s="2" t="s">
         <v>256</v>
       </c>
       <c r="C252" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="253" ht="18.75" spans="1:3">
       <c r="A253" s="2">
-        <v>6056000030</v>
+        <v>6056000029</v>
       </c>
       <c r="B253" s="2" t="s">
         <v>257</v>
       </c>
       <c r="C253" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="254" ht="18.75" spans="1:3">
       <c r="A254" s="2">
-        <v>6056000031</v>
+        <v>6056000030</v>
       </c>
       <c r="B254" s="2" t="s">
         <v>258</v>
       </c>
       <c r="C254" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="255" ht="18.75" spans="1:3">
       <c r="A255" s="2">
-        <v>6056000032</v>
+        <v>6056000031</v>
       </c>
       <c r="B255" s="2" t="s">
         <v>259</v>
       </c>
       <c r="C255" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="256" ht="18.75" spans="1:3">
       <c r="A256" s="2">
-        <v>6056000033</v>
+        <v>6056000032</v>
       </c>
       <c r="B256" s="2" t="s">
         <v>260</v>
       </c>
       <c r="C256" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="257" ht="18.75" spans="1:3">
       <c r="A257" s="2">
-        <v>6056000034</v>
+        <v>6056000033</v>
       </c>
       <c r="B257" s="2" t="s">
         <v>261</v>
       </c>
       <c r="C257" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="258" ht="18.75" spans="1:3">
       <c r="A258" s="2">
-        <v>6056000035</v>
+        <v>6056000034</v>
       </c>
       <c r="B258" s="2" t="s">
         <v>262</v>
       </c>
       <c r="C258" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="259" ht="18.75" spans="1:3">
       <c r="A259" s="2">
-        <v>6056000036</v>
+        <v>6056000035</v>
       </c>
       <c r="B259" s="2" t="s">
         <v>263</v>
       </c>
       <c r="C259" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="260" ht="18.75" spans="1:3">
       <c r="A260" s="2">
-        <v>6056000037</v>
+        <v>6056000036</v>
       </c>
       <c r="B260" s="2" t="s">
         <v>264</v>
       </c>
       <c r="C260" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="261" ht="18.75" spans="1:3">
       <c r="A261" s="2">
-        <v>6056000038</v>
+        <v>6056000037</v>
       </c>
       <c r="B261" s="2" t="s">
         <v>265</v>
       </c>
       <c r="C261" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="262" ht="18.75" spans="1:3">
       <c r="A262" s="2">
-        <v>6056000039</v>
+        <v>6056000038</v>
       </c>
       <c r="B262" s="2" t="s">
         <v>266</v>
       </c>
       <c r="C262" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="263" ht="18.75" spans="1:3">
       <c r="A263" s="2">
-        <v>6056000040</v>
+        <v>6056000039</v>
       </c>
       <c r="B263" s="2" t="s">
-        <v>226</v>
+        <v>267</v>
       </c>
       <c r="C263" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="264" ht="18.75" spans="1:3">
       <c r="A264" s="2">
-        <v>6056000041</v>
+        <v>6056000040</v>
       </c>
       <c r="B264" s="2" t="s">
-        <v>267</v>
+        <v>227</v>
       </c>
       <c r="C264" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="265" ht="18.75" spans="1:3">
       <c r="A265" s="2">
-        <v>6056000042</v>
+        <v>6056000041</v>
       </c>
       <c r="B265" s="2" t="s">
         <v>268</v>
       </c>
       <c r="C265" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="266" ht="18.75" spans="1:3">
       <c r="A266" s="2">
-        <v>6056000043</v>
+        <v>6056000042</v>
       </c>
       <c r="B266" s="2" t="s">
         <v>269</v>
       </c>
       <c r="C266" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="267" ht="18.75" spans="1:3">
       <c r="A267" s="2">
-        <v>6056000044</v>
+        <v>6056000043</v>
       </c>
       <c r="B267" s="2" t="s">
         <v>270</v>
       </c>
       <c r="C267" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="268" ht="18.75" spans="1:3">
       <c r="A268" s="2">
-        <v>6056000045</v>
+        <v>6056000044</v>
       </c>
       <c r="B268" s="2" t="s">
         <v>271</v>
       </c>
       <c r="C268" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="269" ht="18.75" spans="1:3">
       <c r="A269" s="2">
-        <v>6056000046</v>
+        <v>6056000045</v>
       </c>
       <c r="B269" s="2" t="s">
         <v>272</v>
       </c>
       <c r="C269" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="270" ht="18.75" spans="1:3">
       <c r="A270" s="2">
-        <v>6056000047</v>
+        <v>6056000046</v>
       </c>
       <c r="B270" s="2" t="s">
         <v>273</v>
       </c>
       <c r="C270" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="271" ht="18.75" spans="1:3">
       <c r="A271" s="2">
-        <v>6056000048</v>
+        <v>6056000047</v>
       </c>
       <c r="B271" s="2" t="s">
         <v>274</v>
       </c>
       <c r="C271" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="272" ht="18.75" spans="1:3">
       <c r="A272" s="2">
-        <v>6056000049</v>
+        <v>6056000048</v>
       </c>
       <c r="B272" s="2" t="s">
         <v>275</v>
       </c>
       <c r="C272" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="273" ht="18.75" spans="1:3">
       <c r="A273" s="2">
-        <v>6056000050</v>
+        <v>6056000049</v>
       </c>
       <c r="B273" s="2" t="s">
         <v>276</v>
       </c>
       <c r="C273" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="274" ht="18.75" spans="1:3">
       <c r="A274" s="2">
-        <v>6056000051</v>
+        <v>6056000050</v>
       </c>
       <c r="B274" s="2" t="s">
         <v>277</v>
       </c>
       <c r="C274" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="275" ht="18.75" spans="1:3">
       <c r="A275" s="2">
-        <v>6056000052</v>
+        <v>6056000051</v>
       </c>
       <c r="B275" s="2" t="s">
         <v>278</v>
       </c>
       <c r="C275" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="276" ht="18.75" spans="1:3">
       <c r="A276" s="2">
-        <v>6056000053</v>
+        <v>6056000052</v>
       </c>
       <c r="B276" s="2" t="s">
         <v>279</v>
       </c>
       <c r="C276" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="277" ht="18.75" spans="1:3">
       <c r="A277" s="2">
-        <v>6056000054</v>
+        <v>6056000053</v>
       </c>
       <c r="B277" s="2" t="s">
         <v>280</v>
       </c>
       <c r="C277" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="278" ht="18.75" spans="1:3">
       <c r="A278" s="2">
-        <v>6056000055</v>
+        <v>6056000054</v>
       </c>
       <c r="B278" s="2" t="s">
         <v>281</v>
       </c>
       <c r="C278" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="279" ht="18.75" spans="1:3">
       <c r="A279" s="2">
-        <v>6056000056</v>
+        <v>6056000055</v>
       </c>
       <c r="B279" s="2" t="s">
         <v>282</v>
       </c>
       <c r="C279" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="280" ht="18.75" spans="1:3">
       <c r="A280" s="2">
-        <v>6056000057</v>
+        <v>6056000056</v>
       </c>
       <c r="B280" s="2" t="s">
         <v>283</v>
       </c>
       <c r="C280" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="281" ht="18.75" spans="1:3">
       <c r="A281" s="2">
-        <v>6056000058</v>
+        <v>6056000057</v>
       </c>
       <c r="B281" s="2" t="s">
         <v>284</v>
       </c>
       <c r="C281" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="282" ht="18.75" spans="1:3">
       <c r="A282" s="2">
-        <v>6056000059</v>
+        <v>6056000058</v>
       </c>
       <c r="B282" s="2" t="s">
         <v>285</v>
       </c>
       <c r="C282" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="283" ht="18.75" spans="1:3">
       <c r="A283" s="2">
-        <v>6080000001</v>
+        <v>6056000059</v>
       </c>
       <c r="B283" s="2" t="s">
         <v>286</v>
       </c>
       <c r="C283" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="284" ht="18.75" spans="1:3">
       <c r="A284" s="2">
-        <v>6080000002</v>
+        <v>6080000001</v>
       </c>
       <c r="B284" s="2" t="s">
         <v>287</v>
       </c>
       <c r="C284" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="285" ht="18.75" spans="1:3">
       <c r="A285" s="2">
-        <v>6080000003</v>
+        <v>6080000002</v>
       </c>
       <c r="B285" s="2" t="s">
         <v>288</v>
       </c>
       <c r="C285" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="286" ht="18.75" spans="1:3">
       <c r="A286" s="2">
-        <v>6080000004</v>
+        <v>6080000003</v>
       </c>
       <c r="B286" s="2" t="s">
         <v>289</v>
       </c>
       <c r="C286" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="287" ht="18.75" spans="1:3">
       <c r="A287" s="2">
-        <v>6080000005</v>
+        <v>6080000004</v>
       </c>
       <c r="B287" s="2" t="s">
         <v>290</v>
       </c>
       <c r="C287" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="288" ht="18.75" spans="1:3">
-      <c r="A288" s="7">
+      <c r="A288" s="2">
+        <v>6080000005</v>
+      </c>
+      <c r="B288" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="C288" s="2" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="289" ht="18.75" spans="1:3">
+      <c r="A289" s="7">
         <v>6140000000</v>
       </c>
-      <c r="B288" s="7" t="s">
-        <v>291</v>
-      </c>
-      <c r="C288" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="289" ht="18.75" spans="1:3">
-      <c r="A289" s="2">
-        <v>6220000000</v>
-      </c>
-      <c r="B289" s="2" t="s">
+      <c r="B289" s="7" t="s">
         <v>292</v>
       </c>
       <c r="C289" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="290" ht="18.75" spans="1:3">
       <c r="A290" s="2">
-        <v>6223000001</v>
+        <v>6220000000</v>
       </c>
       <c r="B290" s="2" t="s">
         <v>293</v>
       </c>
       <c r="C290" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="291" ht="18.75" spans="1:3">
       <c r="A291" s="2">
-        <v>6223000002</v>
+        <v>6223000001</v>
       </c>
       <c r="B291" s="2" t="s">
         <v>294</v>
       </c>
       <c r="C291" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="292" ht="18.75" spans="1:3">
       <c r="A292" s="2">
-        <v>6223000003</v>
+        <v>6223000002</v>
       </c>
       <c r="B292" s="2" t="s">
         <v>295</v>
       </c>
       <c r="C292" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="293" ht="18.75" spans="1:3">
       <c r="A293" s="2">
-        <v>6223000004</v>
+        <v>6223000003</v>
       </c>
       <c r="B293" s="2" t="s">
         <v>296</v>
       </c>
       <c r="C293" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="294" ht="18.75" spans="1:3">
       <c r="A294" s="2">
-        <v>6223000005</v>
+        <v>6223000004</v>
       </c>
       <c r="B294" s="2" t="s">
         <v>297</v>
       </c>
       <c r="C294" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="295" ht="18.75" spans="1:3">
       <c r="A295" s="2">
-        <v>6223000006</v>
+        <v>6223000005</v>
       </c>
       <c r="B295" s="2" t="s">
         <v>298</v>
       </c>
       <c r="C295" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="296" ht="18.75" spans="1:3">
       <c r="A296" s="2">
-        <v>6223000007</v>
+        <v>6223000006</v>
       </c>
       <c r="B296" s="2" t="s">
         <v>299</v>
       </c>
       <c r="C296" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="297" ht="18.75" spans="1:3">
       <c r="A297" s="2">
-        <v>6223000008</v>
+        <v>6223000007</v>
       </c>
       <c r="B297" s="2" t="s">
         <v>300</v>
       </c>
       <c r="C297" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="298" ht="18.75" spans="1:3">
       <c r="A298" s="2">
-        <v>6223000009</v>
+        <v>6223000008</v>
       </c>
       <c r="B298" s="2" t="s">
         <v>301</v>
       </c>
       <c r="C298" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="299" ht="18.75" spans="1:3">
       <c r="A299" s="2">
-        <v>6240000000</v>
+        <v>6223000009</v>
       </c>
       <c r="B299" s="2" t="s">
         <v>302</v>
       </c>
       <c r="C299" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="300" ht="18.75" spans="1:3">
       <c r="A300" s="2">
-        <v>6240000001</v>
+        <v>6240000000</v>
       </c>
       <c r="B300" s="2" t="s">
         <v>303</v>
       </c>
       <c r="C300" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="301" ht="18.75" spans="1:3">
       <c r="A301" s="2">
-        <v>6240000002</v>
+        <v>6240000001</v>
       </c>
       <c r="B301" s="2" t="s">
         <v>304</v>
       </c>
       <c r="C301" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="302" ht="18.75" spans="1:3">
       <c r="A302" s="2">
-        <v>6240000003</v>
+        <v>6240000002</v>
       </c>
       <c r="B302" s="2" t="s">
         <v>305</v>
       </c>
       <c r="C302" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="303" ht="18.75" spans="1:3">
       <c r="A303" s="2">
-        <v>6240000004</v>
+        <v>6240000003</v>
       </c>
       <c r="B303" s="2" t="s">
         <v>306</v>
       </c>
       <c r="C303" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="304" ht="18.75" spans="1:3">
       <c r="A304" s="2">
-        <v>6240000005</v>
+        <v>6240000004</v>
       </c>
       <c r="B304" s="2" t="s">
         <v>307</v>
       </c>
       <c r="C304" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="305" ht="18.75" spans="1:3">
       <c r="A305" s="2">
-        <v>6240000006</v>
+        <v>6240000005</v>
       </c>
       <c r="B305" s="2" t="s">
         <v>308</v>
       </c>
       <c r="C305" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="306" ht="18.75" spans="1:3">
       <c r="A306" s="2">
-        <v>6240000007</v>
+        <v>6240000006</v>
       </c>
       <c r="B306" s="2" t="s">
         <v>309</v>
       </c>
       <c r="C306" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="307" ht="18.75" spans="1:3">
       <c r="A307" s="2">
-        <v>6240000008</v>
+        <v>6240000007</v>
       </c>
       <c r="B307" s="2" t="s">
         <v>310</v>
       </c>
       <c r="C307" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="308" ht="18.75" spans="1:3">
       <c r="A308" s="2">
-        <v>6240000009</v>
+        <v>6240000008</v>
       </c>
       <c r="B308" s="2" t="s">
         <v>311</v>
       </c>
       <c r="C308" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="309" ht="18.75" spans="1:3">
       <c r="A309" s="2">
-        <v>6288000000</v>
+        <v>6240000009</v>
       </c>
       <c r="B309" s="2" t="s">
         <v>312</v>
       </c>
       <c r="C309" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="310" ht="18.75" spans="1:3">
       <c r="A310" s="2">
-        <v>6384000001</v>
+        <v>6288000000</v>
       </c>
       <c r="B310" s="2" t="s">
         <v>313</v>
       </c>
       <c r="C310" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="311" ht="18.75" spans="1:3">
       <c r="A311" s="2">
-        <v>6384000002</v>
+        <v>6384000001</v>
       </c>
       <c r="B311" s="2" t="s">
         <v>314</v>
       </c>
       <c r="C311" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="312" ht="18.75" spans="1:3">
       <c r="A312" s="2">
-        <v>6500000000</v>
+        <v>6384000002</v>
       </c>
       <c r="B312" s="2" t="s">
         <v>315</v>
       </c>
       <c r="C312" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="313" ht="18.75" spans="1:3">
       <c r="A313" s="2">
-        <v>6620000000</v>
+        <v>6500000000</v>
       </c>
       <c r="B313" s="2" t="s">
         <v>316</v>
       </c>
       <c r="C313" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="314" ht="18.75" spans="1:3">
       <c r="A314" s="2">
-        <v>6621000001</v>
+        <v>6620000000</v>
       </c>
       <c r="B314" s="2" t="s">
         <v>317</v>
       </c>
       <c r="C314" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="315" ht="18.75" spans="1:3">
       <c r="A315" s="2">
-        <v>6621000002</v>
+        <v>6621000001</v>
       </c>
       <c r="B315" s="2" t="s">
         <v>318</v>
       </c>
       <c r="C315" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="316" ht="18.75" spans="1:3">
       <c r="A316" s="2">
-        <v>6631000000</v>
+        <v>6621000002</v>
       </c>
       <c r="B316" s="2" t="s">
         <v>319</v>
       </c>
       <c r="C316" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="317" ht="18.75" spans="1:3">
       <c r="A317" s="2">
-        <v>6662000000</v>
+        <v>6631000000</v>
       </c>
       <c r="B317" s="2" t="s">
         <v>320</v>
       </c>
       <c r="C317" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="318" ht="18.75" spans="1:3">
       <c r="A318" s="2">
-        <v>6672000000</v>
+        <v>6662000000</v>
       </c>
       <c r="B318" s="2" t="s">
         <v>321</v>
       </c>
       <c r="C318" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="319" ht="18.75" spans="1:3">
       <c r="A319" s="2">
-        <v>6672000001</v>
+        <v>6672000000</v>
       </c>
       <c r="B319" s="2" t="s">
         <v>322</v>
       </c>
       <c r="C319" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="320" ht="18.75" spans="1:3">
       <c r="A320" s="2">
-        <v>6672000002</v>
+        <v>6672000001</v>
       </c>
       <c r="B320" s="2" t="s">
         <v>323</v>
       </c>
       <c r="C320" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="321" ht="18.75" spans="1:3">
       <c r="A321" s="2">
-        <v>6672000003</v>
+        <v>6672000002</v>
       </c>
       <c r="B321" s="2" t="s">
         <v>324</v>
       </c>
       <c r="C321" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="322" ht="18.75" spans="1:3">
       <c r="A322" s="2">
-        <v>6730000000</v>
+        <v>6672000003</v>
       </c>
       <c r="B322" s="2" t="s">
         <v>325</v>
       </c>
       <c r="C322" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="323" ht="18.75" spans="1:3">
       <c r="A323" s="2">
-        <v>6760000000</v>
+        <v>6730000000</v>
       </c>
       <c r="B323" s="2" t="s">
         <v>326</v>
       </c>
       <c r="C323" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="324" ht="18.75" spans="1:3">
       <c r="A324" s="2">
-        <v>6810000000</v>
+        <v>6760000000</v>
       </c>
       <c r="B324" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C324" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="325" ht="18.75" spans="1:3">
       <c r="A325" s="2">
-        <v>7010000001</v>
+        <v>6810000000</v>
       </c>
       <c r="B325" s="2" t="s">
         <v>328</v>
       </c>
       <c r="C325" s="2" t="s">
-        <v>329</v>
+        <v>162</v>
       </c>
     </row>
     <row r="326" ht="18.75" spans="1:3">
       <c r="A326" s="2">
-        <v>7010000002</v>
+        <v>7010000001</v>
       </c>
       <c r="B326" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="C326" s="2" t="s">
         <v>330</v>
-      </c>
-      <c r="C326" s="2" t="s">
-        <v>329</v>
       </c>
     </row>
     <row r="327" ht="18.75" spans="1:3">
       <c r="A327" s="2">
-        <v>7010000003</v>
+        <v>7010000002</v>
       </c>
       <c r="B327" s="2" t="s">
         <v>331</v>
       </c>
       <c r="C327" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="328" ht="18.75" spans="1:3">
       <c r="A328" s="2">
-        <v>7010000004</v>
+        <v>7010000003</v>
       </c>
       <c r="B328" s="2" t="s">
         <v>332</v>
       </c>
       <c r="C328" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="329" ht="18.75" spans="1:3">
       <c r="A329" s="2">
-        <v>7010000005</v>
+        <v>7010000004</v>
       </c>
       <c r="B329" s="2" t="s">
         <v>333</v>
       </c>
       <c r="C329" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="330" ht="18.75" spans="1:3">
       <c r="A330" s="2">
-        <v>7010000006</v>
+        <v>7010000005</v>
       </c>
       <c r="B330" s="2" t="s">
         <v>334</v>
       </c>
       <c r="C330" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="331" ht="18.75" spans="1:3">
       <c r="A331" s="2">
-        <v>7010000007</v>
+        <v>7010000006</v>
       </c>
       <c r="B331" s="2" t="s">
         <v>335</v>
       </c>
       <c r="C331" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="332" ht="18.75" spans="1:3">
       <c r="A332" s="2">
-        <v>7010000008</v>
+        <v>7010000007</v>
       </c>
       <c r="B332" s="2" t="s">
         <v>336</v>
       </c>
       <c r="C332" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="333" ht="18.75" spans="1:3">
       <c r="A333" s="2">
-        <v>7010000009</v>
+        <v>7010000008</v>
       </c>
       <c r="B333" s="2" t="s">
         <v>337</v>
       </c>
       <c r="C333" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="334" ht="18.75" spans="1:3">
       <c r="A334" s="2">
-        <v>7010000010</v>
+        <v>7010000009</v>
       </c>
       <c r="B334" s="2" t="s">
         <v>338</v>
       </c>
       <c r="C334" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="335" ht="18.75" spans="1:3">
       <c r="A335" s="2">
-        <v>7010000011</v>
+        <v>7010000010</v>
       </c>
       <c r="B335" s="2" t="s">
         <v>339</v>
       </c>
       <c r="C335" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="336" ht="18.75" spans="1:3">
       <c r="A336" s="2">
-        <v>7010000012</v>
+        <v>7010000011</v>
       </c>
       <c r="B336" s="2" t="s">
         <v>340</v>
       </c>
       <c r="C336" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="337" ht="18.75" spans="1:3">
       <c r="A337" s="2">
-        <v>7060000000</v>
+        <v>7010000012</v>
       </c>
       <c r="B337" s="2" t="s">
         <v>341</v>
       </c>
       <c r="C337" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="338" ht="18.75" spans="1:3">
       <c r="A338" s="2">
-        <v>7588000000</v>
+        <v>7060000000</v>
       </c>
       <c r="B338" s="2" t="s">
         <v>342</v>
       </c>
       <c r="C338" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="339" ht="18.75" spans="1:3">
       <c r="A339" s="2">
-        <v>7760000000</v>
+        <v>7588000000</v>
       </c>
       <c r="B339" s="2" t="s">
         <v>343</v>
       </c>
       <c r="C339" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="340" ht="18.75" spans="1:3">
       <c r="A340" s="2">
-        <v>7870000000</v>
+        <v>7760000000</v>
       </c>
       <c r="B340" s="2" t="s">
         <v>344</v>
       </c>
       <c r="C340" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="341" ht="18.75" spans="1:3">
-      <c r="A341" s="8">
+      <c r="A341" s="2">
+        <v>7870000000</v>
+      </c>
+      <c r="B341" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="C341" s="2" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="342" ht="18.75" spans="1:3">
+      <c r="A342" s="8">
         <v>8910000000</v>
       </c>
-      <c r="B341" s="8" t="s">
-        <v>345</v>
-      </c>
-      <c r="C341" s="8" t="s">
-        <v>161</v>
+      <c r="B342" s="8" t="s">
+        <v>346</v>
+      </c>
+      <c r="C342" s="8" t="s">
+        <v>162</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
derier commit apres suppression de CB
</commit_message>
<xml_diff>
--- a/public/PLAN.xlsx
+++ b/public/PLAN.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="708" uniqueCount="363">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="710" uniqueCount="364">
   <si>
     <t>Comptes</t>
   </si>
@@ -930,6 +930,9 @@
   </si>
   <si>
     <t>Achat barre de 10</t>
+  </si>
+  <si>
+    <t>Achat Contre-plaquet</t>
   </si>
   <si>
     <t>Achat  enveloppe sac( emballage)</t>
@@ -2171,7 +2174,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C358"/>
+  <dimension ref="A1:C359"/>
   <sheetFormatPr defaultColWidth="11.4571428571429" defaultRowHeight="15" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="19.4571428571429" customWidth="1"/>
@@ -5430,7 +5433,7 @@
     </row>
     <row r="298" ht="18.75" spans="1:3">
       <c r="A298" s="2">
-        <v>6080000001</v>
+        <v>6056000061</v>
       </c>
       <c r="B298" s="2" t="s">
         <v>301</v>
@@ -5441,7 +5444,7 @@
     </row>
     <row r="299" ht="18.75" spans="1:3">
       <c r="A299" s="2">
-        <v>6080000002</v>
+        <v>6080000001</v>
       </c>
       <c r="B299" s="2" t="s">
         <v>302</v>
@@ -5452,7 +5455,7 @@
     </row>
     <row r="300" ht="18.75" spans="1:3">
       <c r="A300" s="2">
-        <v>6080000003</v>
+        <v>6080000002</v>
       </c>
       <c r="B300" s="2" t="s">
         <v>303</v>
@@ -5463,7 +5466,7 @@
     </row>
     <row r="301" ht="18.75" spans="1:3">
       <c r="A301" s="2">
-        <v>6080000004</v>
+        <v>6080000003</v>
       </c>
       <c r="B301" s="2" t="s">
         <v>304</v>
@@ -5474,7 +5477,7 @@
     </row>
     <row r="302" ht="18.75" spans="1:3">
       <c r="A302" s="2">
-        <v>6080000005</v>
+        <v>6080000004</v>
       </c>
       <c r="B302" s="2" t="s">
         <v>305</v>
@@ -5484,21 +5487,21 @@
       </c>
     </row>
     <row r="303" ht="18.75" spans="1:3">
-      <c r="A303" s="7">
+      <c r="A303" s="2">
+        <v>6080000005</v>
+      </c>
+      <c r="B303" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="C303" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="304" ht="18.75" spans="1:3">
+      <c r="A304" s="7">
         <v>6140000000</v>
       </c>
-      <c r="B303" s="7" t="s">
-        <v>306</v>
-      </c>
-      <c r="C303" s="2" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="304" ht="18.75" spans="1:3">
-      <c r="A304" s="2">
-        <v>6220000000</v>
-      </c>
-      <c r="B304" s="2" t="s">
+      <c r="B304" s="7" t="s">
         <v>307</v>
       </c>
       <c r="C304" s="2" t="s">
@@ -5507,7 +5510,7 @@
     </row>
     <row r="305" ht="18.75" spans="1:3">
       <c r="A305" s="2">
-        <v>6223000001</v>
+        <v>6220000000</v>
       </c>
       <c r="B305" s="2" t="s">
         <v>308</v>
@@ -5518,7 +5521,7 @@
     </row>
     <row r="306" ht="18.75" spans="1:3">
       <c r="A306" s="2">
-        <v>6223000002</v>
+        <v>6223000001</v>
       </c>
       <c r="B306" s="2" t="s">
         <v>309</v>
@@ -5529,7 +5532,7 @@
     </row>
     <row r="307" ht="18.75" spans="1:3">
       <c r="A307" s="2">
-        <v>6223000003</v>
+        <v>6223000002</v>
       </c>
       <c r="B307" s="2" t="s">
         <v>310</v>
@@ -5540,7 +5543,7 @@
     </row>
     <row r="308" ht="18.75" spans="1:3">
       <c r="A308" s="2">
-        <v>6223000004</v>
+        <v>6223000003</v>
       </c>
       <c r="B308" s="2" t="s">
         <v>311</v>
@@ -5551,7 +5554,7 @@
     </row>
     <row r="309" ht="18.75" spans="1:3">
       <c r="A309" s="2">
-        <v>6223000005</v>
+        <v>6223000004</v>
       </c>
       <c r="B309" s="2" t="s">
         <v>312</v>
@@ -5562,7 +5565,7 @@
     </row>
     <row r="310" ht="18.75" spans="1:3">
       <c r="A310" s="2">
-        <v>6223000006</v>
+        <v>6223000005</v>
       </c>
       <c r="B310" s="2" t="s">
         <v>313</v>
@@ -5573,7 +5576,7 @@
     </row>
     <row r="311" ht="18.75" spans="1:3">
       <c r="A311" s="2">
-        <v>6223000007</v>
+        <v>6223000006</v>
       </c>
       <c r="B311" s="2" t="s">
         <v>314</v>
@@ -5584,7 +5587,7 @@
     </row>
     <row r="312" ht="18.75" spans="1:3">
       <c r="A312" s="2">
-        <v>6223000008</v>
+        <v>6223000007</v>
       </c>
       <c r="B312" s="2" t="s">
         <v>315</v>
@@ -5595,7 +5598,7 @@
     </row>
     <row r="313" ht="18.75" spans="1:3">
       <c r="A313" s="2">
-        <v>6223000009</v>
+        <v>6223000008</v>
       </c>
       <c r="B313" s="2" t="s">
         <v>316</v>
@@ -5606,7 +5609,7 @@
     </row>
     <row r="314" ht="18.75" spans="1:3">
       <c r="A314" s="2">
-        <v>6240000000</v>
+        <v>6223000009</v>
       </c>
       <c r="B314" s="2" t="s">
         <v>317</v>
@@ -5617,7 +5620,7 @@
     </row>
     <row r="315" ht="18.75" spans="1:3">
       <c r="A315" s="2">
-        <v>6240000001</v>
+        <v>6240000000</v>
       </c>
       <c r="B315" s="2" t="s">
         <v>318</v>
@@ -5628,7 +5631,7 @@
     </row>
     <row r="316" ht="18.75" spans="1:3">
       <c r="A316" s="2">
-        <v>6240000002</v>
+        <v>6240000001</v>
       </c>
       <c r="B316" s="2" t="s">
         <v>319</v>
@@ -5639,7 +5642,7 @@
     </row>
     <row r="317" ht="18.75" spans="1:3">
       <c r="A317" s="2">
-        <v>6240000003</v>
+        <v>6240000002</v>
       </c>
       <c r="B317" s="2" t="s">
         <v>320</v>
@@ -5650,7 +5653,7 @@
     </row>
     <row r="318" ht="18.75" spans="1:3">
       <c r="A318" s="2">
-        <v>6240000004</v>
+        <v>6240000003</v>
       </c>
       <c r="B318" s="2" t="s">
         <v>321</v>
@@ -5661,7 +5664,7 @@
     </row>
     <row r="319" ht="18.75" spans="1:3">
       <c r="A319" s="2">
-        <v>6240000005</v>
+        <v>6240000004</v>
       </c>
       <c r="B319" s="2" t="s">
         <v>322</v>
@@ -5672,7 +5675,7 @@
     </row>
     <row r="320" ht="18.75" spans="1:3">
       <c r="A320" s="2">
-        <v>6240000006</v>
+        <v>6240000005</v>
       </c>
       <c r="B320" s="2" t="s">
         <v>323</v>
@@ -5683,7 +5686,7 @@
     </row>
     <row r="321" ht="18.75" spans="1:3">
       <c r="A321" s="2">
-        <v>6240000007</v>
+        <v>6240000006</v>
       </c>
       <c r="B321" s="2" t="s">
         <v>324</v>
@@ -5694,7 +5697,7 @@
     </row>
     <row r="322" ht="18.75" spans="1:3">
       <c r="A322" s="2">
-        <v>6240000008</v>
+        <v>6240000007</v>
       </c>
       <c r="B322" s="2" t="s">
         <v>325</v>
@@ -5705,7 +5708,7 @@
     </row>
     <row r="323" ht="18.75" spans="1:3">
       <c r="A323" s="2">
-        <v>6240000009</v>
+        <v>6240000008</v>
       </c>
       <c r="B323" s="2" t="s">
         <v>326</v>
@@ -5716,7 +5719,7 @@
     </row>
     <row r="324" ht="18.75" spans="1:3">
       <c r="A324" s="2">
-        <v>6240000010</v>
+        <v>6240000009</v>
       </c>
       <c r="B324" s="2" t="s">
         <v>327</v>
@@ -5727,7 +5730,7 @@
     </row>
     <row r="325" ht="18.75" spans="1:3">
       <c r="A325" s="2">
-        <v>6288000000</v>
+        <v>6240000010</v>
       </c>
       <c r="B325" s="2" t="s">
         <v>328</v>
@@ -5738,7 +5741,7 @@
     </row>
     <row r="326" ht="18.75" spans="1:3">
       <c r="A326" s="2">
-        <v>6384000001</v>
+        <v>6288000000</v>
       </c>
       <c r="B326" s="2" t="s">
         <v>329</v>
@@ -5749,7 +5752,7 @@
     </row>
     <row r="327" ht="18.75" spans="1:3">
       <c r="A327" s="2">
-        <v>6384000002</v>
+        <v>6384000001</v>
       </c>
       <c r="B327" s="2" t="s">
         <v>330</v>
@@ -5760,7 +5763,7 @@
     </row>
     <row r="328" ht="18.75" spans="1:3">
       <c r="A328" s="2">
-        <v>6500000000</v>
+        <v>6384000002</v>
       </c>
       <c r="B328" s="2" t="s">
         <v>331</v>
@@ -5771,7 +5774,7 @@
     </row>
     <row r="329" ht="18.75" spans="1:3">
       <c r="A329" s="2">
-        <v>6620000000</v>
+        <v>6500000000</v>
       </c>
       <c r="B329" s="2" t="s">
         <v>332</v>
@@ -5782,7 +5785,7 @@
     </row>
     <row r="330" ht="18.75" spans="1:3">
       <c r="A330" s="2">
-        <v>6621000001</v>
+        <v>6620000000</v>
       </c>
       <c r="B330" s="2" t="s">
         <v>333</v>
@@ -5793,7 +5796,7 @@
     </row>
     <row r="331" ht="18.75" spans="1:3">
       <c r="A331" s="2">
-        <v>6621000002</v>
+        <v>6621000001</v>
       </c>
       <c r="B331" s="2" t="s">
         <v>334</v>
@@ -5804,7 +5807,7 @@
     </row>
     <row r="332" ht="18.75" spans="1:3">
       <c r="A332" s="2">
-        <v>6631000000</v>
+        <v>6621000002</v>
       </c>
       <c r="B332" s="2" t="s">
         <v>335</v>
@@ -5815,7 +5818,7 @@
     </row>
     <row r="333" ht="18.75" spans="1:3">
       <c r="A333" s="2">
-        <v>6662000000</v>
+        <v>6631000000</v>
       </c>
       <c r="B333" s="2" t="s">
         <v>336</v>
@@ -5826,7 +5829,7 @@
     </row>
     <row r="334" ht="18.75" spans="1:3">
       <c r="A334" s="2">
-        <v>6672000000</v>
+        <v>6662000000</v>
       </c>
       <c r="B334" s="2" t="s">
         <v>337</v>
@@ -5837,7 +5840,7 @@
     </row>
     <row r="335" ht="18.75" spans="1:3">
       <c r="A335" s="2">
-        <v>6672000001</v>
+        <v>6672000000</v>
       </c>
       <c r="B335" s="2" t="s">
         <v>338</v>
@@ -5848,7 +5851,7 @@
     </row>
     <row r="336" ht="18.75" spans="1:3">
       <c r="A336" s="2">
-        <v>6672000002</v>
+        <v>6672000001</v>
       </c>
       <c r="B336" s="2" t="s">
         <v>339</v>
@@ -5859,7 +5862,7 @@
     </row>
     <row r="337" ht="18.75" spans="1:3">
       <c r="A337" s="2">
-        <v>6672000003</v>
+        <v>6672000002</v>
       </c>
       <c r="B337" s="2" t="s">
         <v>340</v>
@@ -5870,7 +5873,7 @@
     </row>
     <row r="338" ht="18.75" spans="1:3">
       <c r="A338" s="2">
-        <v>6730000000</v>
+        <v>6672000003</v>
       </c>
       <c r="B338" s="2" t="s">
         <v>341</v>
@@ -5881,7 +5884,7 @@
     </row>
     <row r="339" ht="18.75" spans="1:3">
       <c r="A339" s="2">
-        <v>6760000000</v>
+        <v>6730000000</v>
       </c>
       <c r="B339" s="2" t="s">
         <v>342</v>
@@ -5892,7 +5895,7 @@
     </row>
     <row r="340" ht="18.75" spans="1:3">
       <c r="A340" s="2">
-        <v>6810000000</v>
+        <v>6760000000</v>
       </c>
       <c r="B340" s="2" t="s">
         <v>343</v>
@@ -5903,199 +5906,210 @@
     </row>
     <row r="341" ht="18.75" spans="1:3">
       <c r="A341" s="2">
-        <v>7010000001</v>
+        <v>6810000000</v>
       </c>
       <c r="B341" s="2" t="s">
         <v>344</v>
       </c>
       <c r="C341" s="2" t="s">
-        <v>345</v>
+        <v>168</v>
       </c>
     </row>
     <row r="342" ht="18.75" spans="1:3">
       <c r="A342" s="2">
-        <v>7010000002</v>
+        <v>7010000001</v>
       </c>
       <c r="B342" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="C342" s="2" t="s">
         <v>346</v>
-      </c>
-      <c r="C342" s="2" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="343" ht="18.75" spans="1:3">
       <c r="A343" s="2">
-        <v>7010000003</v>
+        <v>7010000002</v>
       </c>
       <c r="B343" s="2" t="s">
         <v>347</v>
       </c>
       <c r="C343" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="344" ht="18.75" spans="1:3">
       <c r="A344" s="2">
-        <v>7010000004</v>
+        <v>7010000003</v>
       </c>
       <c r="B344" s="2" t="s">
         <v>348</v>
       </c>
       <c r="C344" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="345" ht="18.75" spans="1:3">
       <c r="A345" s="2">
-        <v>7010000005</v>
+        <v>7010000004</v>
       </c>
       <c r="B345" s="2" t="s">
         <v>349</v>
       </c>
       <c r="C345" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="346" ht="18.75" spans="1:3">
       <c r="A346" s="2">
-        <v>7010000006</v>
+        <v>7010000005</v>
       </c>
       <c r="B346" s="2" t="s">
         <v>350</v>
       </c>
       <c r="C346" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="347" ht="18.75" spans="1:3">
       <c r="A347" s="2">
-        <v>7010000007</v>
+        <v>7010000006</v>
       </c>
       <c r="B347" s="2" t="s">
         <v>351</v>
       </c>
       <c r="C347" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="348" ht="18.75" spans="1:3">
       <c r="A348" s="2">
-        <v>7010000008</v>
+        <v>7010000007</v>
       </c>
       <c r="B348" s="2" t="s">
         <v>352</v>
       </c>
       <c r="C348" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="349" ht="18.75" spans="1:3">
       <c r="A349" s="2">
-        <v>7010000009</v>
+        <v>7010000008</v>
       </c>
       <c r="B349" s="2" t="s">
         <v>353</v>
       </c>
       <c r="C349" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="350" ht="18.75" spans="1:3">
       <c r="A350" s="2">
-        <v>7010000010</v>
+        <v>7010000009</v>
       </c>
       <c r="B350" s="2" t="s">
         <v>354</v>
       </c>
       <c r="C350" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="351" ht="18.75" spans="1:3">
       <c r="A351" s="2">
-        <v>7010000011</v>
+        <v>7010000010</v>
       </c>
       <c r="B351" s="2" t="s">
         <v>355</v>
       </c>
       <c r="C351" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="352" ht="18.75" spans="1:3">
       <c r="A352" s="2">
-        <v>7010000012</v>
+        <v>7010000011</v>
       </c>
       <c r="B352" s="2" t="s">
         <v>356</v>
       </c>
       <c r="C352" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="353" ht="18.75" spans="1:3">
       <c r="A353" s="2">
-        <v>7010000013</v>
+        <v>7010000012</v>
       </c>
       <c r="B353" s="2" t="s">
         <v>357</v>
       </c>
       <c r="C353" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="354" ht="18.75" spans="1:3">
       <c r="A354" s="2">
-        <v>7060000000</v>
+        <v>7010000013</v>
       </c>
       <c r="B354" s="2" t="s">
         <v>358</v>
       </c>
       <c r="C354" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="355" ht="18.75" spans="1:3">
       <c r="A355" s="2">
-        <v>7588000000</v>
+        <v>7060000000</v>
       </c>
       <c r="B355" s="2" t="s">
         <v>359</v>
       </c>
       <c r="C355" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="356" ht="18.75" spans="1:3">
       <c r="A356" s="2">
-        <v>7760000000</v>
+        <v>7588000000</v>
       </c>
       <c r="B356" s="2" t="s">
         <v>360</v>
       </c>
       <c r="C356" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="357" ht="18.75" spans="1:3">
       <c r="A357" s="2">
-        <v>7870000000</v>
+        <v>7760000000</v>
       </c>
       <c r="B357" s="2" t="s">
         <v>361</v>
       </c>
       <c r="C357" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="358" ht="18.75" spans="1:3">
-      <c r="A358" s="8">
+      <c r="A358" s="2">
+        <v>7870000000</v>
+      </c>
+      <c r="B358" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="C358" s="2" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="359" ht="18.75" spans="1:3">
+      <c r="A359" s="8">
         <v>8910000000</v>
       </c>
-      <c r="B358" s="8" t="s">
-        <v>362</v>
-      </c>
-      <c r="C358" s="8" t="s">
+      <c r="B359" s="8" t="s">
+        <v>363</v>
+      </c>
+      <c r="C359" s="8" t="s">
         <v>168</v>
       </c>
     </row>

</xml_diff>